<commit_message>
Price bound pieces by their reach, and settle the catalogue's moves
A piece whose own move binds it to part of the board is devalued by the
share it can reach: -2 for half, -3 for a quarter, -4 for an eighth or
less. The Private, which moved as the Courtier does, is gone; the
Makruk Pawn promotes to the Courtier. The Silver General, Noble and
Janggi Soldier move as in their own games, and their direction counts
follow. A Janggi Cannon may not jump over a Cannon of either kind.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$W$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$W$41</definedName>
   </definedNames>
   <calcPr calcId="114210"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="136">
   <si>
     <t>Piece Class</t>
   </si>
@@ -416,6 +416,15 @@
   </si>
   <si>
     <t>Restricted to one square in nine (by its leap)</t>
+  </si>
+  <si>
+    <t>Moves one square diagonally, or one square straight forward.</t>
+  </si>
+  <si>
+    <t>Moves one square forward or sideways; in a palace, also diagonally forward along marked palace lines.</t>
+  </si>
+  <si>
+    <t>Must jump over exactly one intervening piece; cannot jump over a Cannon of either kind.</t>
   </si>
 </sst>
 </file>
@@ -808,7 +817,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:W42"/>
+  <dimension ref="A1:W41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="6"/>
@@ -1123,14 +1132,16 @@
         <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>73</v>
+        <v>133</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="H6" s="2" t="s">
         <v>117</v>
       </c>
@@ -1910,7 +1921,7 @@
         <v>85</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
@@ -2058,10 +2069,10 @@
         <v>0</v>
       </c>
       <c r="T22" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="U22" s="2">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
@@ -2422,14 +2433,16 @@
         <v>55</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>92</v>
+        <v>133</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G29" s="2"/>
+      <c r="G29" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="H29" s="2" t="s">
         <v>117</v>
       </c>
@@ -2447,7 +2460,7 @@
         <v>0</v>
       </c>
       <c r="P29" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q29" s="2">
         <v>0</v>
@@ -2462,7 +2475,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
@@ -2516,10 +2529,10 @@
         <v>0</v>
       </c>
       <c r="T30" s="2">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="U30" s="2">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="V30" s="2"/>
       <c r="W30" s="2"/>
@@ -2636,10 +2649,10 @@
         <v>0</v>
       </c>
       <c r="T32" s="2">
-        <v>-2</v>
+        <v>-6</v>
       </c>
       <c r="U32" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="V32" s="2">
         <v>2</v>
@@ -2697,10 +2710,10 @@
         <v>0</v>
       </c>
       <c r="T33" s="2">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="U33" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="V33" s="2"/>
       <c r="W33" s="2"/>
@@ -2754,10 +2767,10 @@
         <v>0</v>
       </c>
       <c r="T34" s="2">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="U34" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="V34" s="2"/>
       <c r="W34" s="2"/>
@@ -2770,7 +2783,7 @@
         <v>62</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>91</v>
+        <v>134</v>
       </c>
       <c r="D35" s="2" t="s">
         <v>105</v>
@@ -2789,7 +2802,7 @@
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K35" s="2">
         <v>1</v>
@@ -2925,10 +2938,10 @@
         <v>0</v>
       </c>
       <c r="T37" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="U37" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V37" s="2"/>
       <c r="W37" s="2"/>
@@ -3024,7 +3037,7 @@
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="2" t="s">
-        <v>130</v>
+        <v>63</v>
       </c>
       <c r="N39" s="2" t="s">
         <v>129</v>
@@ -3055,19 +3068,19 @@
       </c>
       <c r="W39" s="2"/>
     </row>
-    <row r="40" spans="1:23" ht="45" hidden="1">
+    <row r="40" spans="1:23" ht="33.75" hidden="1">
       <c r="A40" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>114</v>
@@ -3102,38 +3115,42 @@
         <v>0</v>
       </c>
       <c r="T40" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="U40" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V40" s="2"/>
-      <c r="W40" s="2"/>
-    </row>
-    <row r="41" spans="1:23" ht="33.75" hidden="1">
+      <c r="W40" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" ht="157.5" hidden="1">
       <c r="A41" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D41" s="2"/>
+        <v>96</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="E41" s="2" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="G41" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="H41" s="2"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K41" s="2">
         <v>1</v>
@@ -3145,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="P41" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q41" s="2">
         <v>0</v>
@@ -3157,77 +3174,18 @@
         <v>0</v>
       </c>
       <c r="T41" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="U41" s="2">
         <v>2</v>
       </c>
       <c r="V41" s="2"/>
       <c r="W41" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:23" ht="157.5" hidden="1">
-      <c r="A42" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H42" s="2"/>
-      <c r="I42" s="2"/>
-      <c r="J42" s="2">
         <v>3</v>
       </c>
-      <c r="K42" s="2">
-        <v>1</v>
-      </c>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2">
-        <v>0</v>
-      </c>
-      <c r="P42" s="2">
-        <v>3</v>
-      </c>
-      <c r="Q42" s="2">
-        <v>0</v>
-      </c>
-      <c r="R42" s="2">
-        <v>0</v>
-      </c>
-      <c r="S42" s="2">
-        <v>0</v>
-      </c>
-      <c r="T42" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U42" s="2">
-        <v>2</v>
-      </c>
-      <c r="V42" s="2"/>
-      <c r="W42" s="2">
-        <v>3</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W42">
+  <autoFilter ref="A1:W41">
     <filterColumn colId="0">
       <filters>
         <filter val="Cavalry / Leaper"/>

</xml_diff>

<commit_message>
Take the designer's re-priced sheet, and settle more of the catalogue
The sheet now computes each value, with the speed bonus counted twice,
and is sorted by value; the catalogue follows it. The Minister and
Courtier are Infantry; the Zebra has no colour restriction, its leap
changing colour every time; the Janggi Cannon keeps the Janggi rule,
neither hopping nor capturing a Cannon of either kind, at -2. Lifts for
the three restrictions without one, and two ways of weighing speed so
that leaps and hops are not doubled, are proposed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -12,12 +12,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$W$41</definedName>
   </definedNames>
-  <calcPr calcId="114210"/>
+  <calcPr calcId="114210" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="133">
   <si>
     <t>Piece Class</t>
   </si>
@@ -217,9 +217,6 @@
     <t>Pawn (Makruk)</t>
   </si>
   <si>
-    <t>Private (Makruk)</t>
-  </si>
-  <si>
     <t>Advisor (Xiangqi)</t>
   </si>
   <si>
@@ -295,9 +292,6 @@
     <t>Moves one square orthogonally forward.</t>
   </si>
   <si>
-    <t>Moves one square diagonally forward.</t>
-  </si>
-  <si>
     <t>Leaps 2+2 squares diagonally.</t>
   </si>
   <si>
@@ -316,9 +310,6 @@
     <t>Must jump over the first intervening piece and land on the immediately adjacent square beyond it.</t>
   </si>
   <si>
-    <t>Must jump over exactly one intervening piece; cannot jump over another Cannon.</t>
-  </si>
-  <si>
     <t>The adjacent square along the two-square leg must be unoccupied.</t>
   </si>
   <si>
@@ -409,9 +400,6 @@
     <t>On reaching the sixth rank</t>
   </si>
   <si>
-    <t>Private</t>
-  </si>
-  <si>
     <t>Moves any number of squares orthogonally, or one square diagonally.</t>
   </si>
   <si>
@@ -425,6 +413,9 @@
   </si>
   <si>
     <t>Must jump over exactly one intervening piece; cannot jump over a Cannon of either kind.</t>
+  </si>
+  <si>
+    <t>Must jump over exactly one intervening piece; may neither jump over nor capture a Cannon of either kind.</t>
   </si>
 </sst>
 </file>
@@ -816,7 +807,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:W41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -896,7 +886,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="33.75" hidden="1">
+    <row r="2" spans="1:23" ht="33.75">
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
@@ -904,18 +894,18 @@
         <v>28</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2">
@@ -946,12 +936,13 @@
         <v>0</v>
       </c>
       <c r="U2" s="2">
-        <v>75</v>
+        <f t="shared" ref="U2:U41" si="0">O2+P2+Q2*2+R2+S2+T2</f>
+        <v>82</v>
       </c>
       <c r="V2" s="2"/>
       <c r="W2" s="2"/>
     </row>
-    <row r="3" spans="1:23" ht="33.75" hidden="1">
+    <row r="3" spans="1:23" ht="33.75">
       <c r="A3" s="5" t="s">
         <v>23</v>
       </c>
@@ -959,17 +950,17 @@
         <v>29</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
@@ -980,7 +971,7 @@
         <v>7</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
@@ -1003,14 +994,15 @@
         <v>-2</v>
       </c>
       <c r="U3" s="2">
-        <v>72</v>
+        <f t="shared" si="0"/>
+        <v>79</v>
       </c>
       <c r="V3" s="2"/>
       <c r="W3" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:23" ht="33.75" hidden="1">
+    <row r="4" spans="1:23" ht="33.75">
       <c r="A4" s="5" t="s">
         <v>23</v>
       </c>
@@ -1018,21 +1010,21 @@
         <v>30</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J4" s="2">
         <v>8</v>
@@ -1062,12 +1054,13 @@
         <v>0</v>
       </c>
       <c r="U4" s="2">
-        <v>71</v>
+        <f t="shared" si="0"/>
+        <v>74</v>
       </c>
       <c r="V4" s="2"/>
       <c r="W4" s="2"/>
     </row>
-    <row r="5" spans="1:23" ht="22.5" hidden="1">
+    <row r="5" spans="1:23" ht="22.5">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
@@ -1075,18 +1068,18 @@
         <v>31</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
@@ -1096,7 +1089,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1119,12 +1112,13 @@
         <v>0</v>
       </c>
       <c r="U5" s="2">
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
       <c r="V5" s="2"/>
       <c r="W5" s="2"/>
     </row>
-    <row r="6" spans="1:23" ht="78.75" hidden="1">
+    <row r="6" spans="1:23" ht="78.75">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -1132,18 +1126,18 @@
         <v>32</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
@@ -1154,10 +1148,10 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="O6" s="2">
         <v>60</v>
@@ -1178,12 +1172,13 @@
         <v>0</v>
       </c>
       <c r="U6" s="2">
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="V6" s="2"/>
       <c r="W6" s="2"/>
     </row>
-    <row r="7" spans="1:23" ht="33.75" hidden="1">
+    <row r="7" spans="1:23" ht="33.75">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
@@ -1191,20 +1186,20 @@
         <v>33</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
@@ -1214,7 +1209,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -1237,6 +1232,7 @@
         <v>-2</v>
       </c>
       <c r="U7" s="2">
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="V7" s="2"/>
@@ -1244,7 +1240,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="33.75" hidden="1">
+    <row r="8" spans="1:23" ht="33.75">
       <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
@@ -1252,18 +1248,18 @@
         <v>34</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
@@ -1294,12 +1290,13 @@
         <v>0</v>
       </c>
       <c r="U8" s="2">
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
       <c r="V8" s="2"/>
       <c r="W8" s="2"/>
     </row>
-    <row r="9" spans="1:23" ht="33.75" hidden="1">
+    <row r="9" spans="1:23" ht="33.75">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -1307,21 +1304,21 @@
         <v>35</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J9" s="2">
         <v>8</v>
@@ -1351,7 +1348,8 @@
         <v>0</v>
       </c>
       <c r="U9" s="2">
-        <v>17</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="V9" s="2"/>
       <c r="W9" s="2"/>
@@ -1364,19 +1362,19 @@
         <v>36</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J10" s="2">
         <v>8</v>
@@ -1406,12 +1404,13 @@
         <v>0</v>
       </c>
       <c r="U10" s="2">
-        <v>16</v>
+        <f t="shared" si="0"/>
+        <v>24</v>
       </c>
       <c r="V10" s="2"/>
       <c r="W10" s="2"/>
     </row>
-    <row r="11" spans="1:23" ht="22.5" hidden="1">
+    <row r="11" spans="1:23" ht="22.5">
       <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
@@ -1419,18 +1418,18 @@
         <v>37</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I11" s="2"/>
       <c r="J11" s="2">
@@ -1461,12 +1460,13 @@
         <v>0</v>
       </c>
       <c r="U11" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="V11" s="2"/>
       <c r="W11" s="2"/>
     </row>
-    <row r="12" spans="1:23" ht="33.75" hidden="1">
+    <row r="12" spans="1:23" ht="22.5">
       <c r="A12" s="5" t="s">
         <v>25</v>
       </c>
@@ -1474,19 +1474,19 @@
         <v>38</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J12" s="2">
         <v>8</v>
@@ -1516,12 +1516,13 @@
         <v>0</v>
       </c>
       <c r="U12" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="V12" s="2"/>
       <c r="W12" s="2"/>
     </row>
-    <row r="13" spans="1:23" ht="33.75" hidden="1">
+    <row r="13" spans="1:23" ht="33.75">
       <c r="A13" s="5" t="s">
         <v>25</v>
       </c>
@@ -1529,19 +1530,19 @@
         <v>39</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J13" s="2">
         <v>8</v>
@@ -1571,12 +1572,13 @@
         <v>0</v>
       </c>
       <c r="U13" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="V13" s="2"/>
       <c r="W13" s="2"/>
     </row>
-    <row r="14" spans="1:23" ht="33.75" hidden="1">
+    <row r="14" spans="1:23" ht="33.75">
       <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
@@ -1584,18 +1586,18 @@
         <v>40</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2">
@@ -1626,12 +1628,13 @@
         <v>0</v>
       </c>
       <c r="U14" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
     </row>
-    <row r="15" spans="1:23" ht="33.75" hidden="1">
+    <row r="15" spans="1:23" ht="33.75">
       <c r="A15" s="5" t="s">
         <v>25</v>
       </c>
@@ -1639,19 +1642,19 @@
         <v>41</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J15" s="2">
         <v>8</v>
@@ -1681,12 +1684,13 @@
         <v>0</v>
       </c>
       <c r="U15" s="2">
-        <v>15</v>
+        <f t="shared" si="0"/>
+        <v>22</v>
       </c>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
     </row>
-    <row r="16" spans="1:23" ht="112.5" hidden="1">
+    <row r="16" spans="1:23" ht="112.5">
       <c r="A16" s="5" t="s">
         <v>27</v>
       </c>
@@ -1694,23 +1698,23 @@
         <v>42</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J16" s="2">
         <v>8</v>
@@ -1740,19 +1744,20 @@
         <v>-1</v>
       </c>
       <c r="U16" s="2">
-        <v>14</v>
+        <f t="shared" si="0"/>
+        <v>21</v>
       </c>
       <c r="V16" s="2">
         <v>3</v>
       </c>
       <c r="W16" s="2"/>
     </row>
-    <row r="17" spans="1:23" ht="22.5">
+    <row r="17" spans="1:23" ht="112.5">
       <c r="A17" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>82</v>
@@ -1760,18 +1765,18 @@
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G17" s="2"/>
+        <v>112</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="H17" s="2"/>
-      <c r="I17" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="I17" s="2"/>
       <c r="J17" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K17" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L17" s="2"/>
       <c r="M17" s="2"/>
@@ -1780,46 +1785,51 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q17" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="R17" s="2">
         <v>0</v>
       </c>
       <c r="S17" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T17" s="2">
         <v>0</v>
       </c>
       <c r="U17" s="2">
-        <v>13</v>
+        <f t="shared" si="0"/>
+        <v>20</v>
       </c>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
     </row>
-    <row r="18" spans="1:23" ht="112.5" hidden="1">
+    <row r="18" spans="1:23" ht="101.25">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D18" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J18" s="2">
         <v>4</v>
       </c>
@@ -1845,35 +1855,36 @@
         <v>2</v>
       </c>
       <c r="T18" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="U18" s="2">
-        <v>13</v>
-      </c>
-      <c r="V18" s="2"/>
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="V18" s="2">
+        <v>3</v>
+      </c>
       <c r="W18" s="2"/>
     </row>
-    <row r="19" spans="1:23" ht="45">
+    <row r="19" spans="1:23" ht="22.5">
       <c r="A19" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="2" t="s">
-        <v>109</v>
-      </c>
+      <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J19" s="2">
         <v>8</v>
@@ -1900,40 +1911,35 @@
         <v>0</v>
       </c>
       <c r="T19" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U19" s="2">
-        <v>12</v>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="V19" s="2"/>
-      <c r="W19" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:23" ht="101.25" hidden="1">
+      <c r="W19" s="2"/>
+    </row>
+    <row r="20" spans="1:23" ht="22.5">
       <c r="A20" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>135</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H20" s="2"/>
-      <c r="I20" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="I20" s="2"/>
       <c r="J20" s="2">
         <v>4</v>
       </c>
@@ -1956,44 +1962,43 @@
         <v>0</v>
       </c>
       <c r="S20" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T20" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U20" s="2">
-        <v>12</v>
-      </c>
-      <c r="V20" s="2">
-        <v>3</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>18</v>
+      </c>
+      <c r="V20" s="2"/>
       <c r="W20" s="2"/>
     </row>
-    <row r="21" spans="1:23" ht="22.5">
+    <row r="21" spans="1:23" ht="45">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J21" s="2">
         <v>8</v>
       </c>
       <c r="K21" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -2005,7 +2010,7 @@
         <v>8</v>
       </c>
       <c r="Q21" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R21" s="2">
         <v>0</v>
@@ -2017,38 +2022,39 @@
         <v>0</v>
       </c>
       <c r="U21" s="2">
-        <v>11</v>
+        <f t="shared" si="0"/>
+        <v>18</v>
       </c>
       <c r="V21" s="2"/>
       <c r="W21" s="2"/>
     </row>
-    <row r="22" spans="1:23" ht="22.5">
+    <row r="22" spans="1:23" ht="45">
       <c r="A22" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="H22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I22" s="2"/>
       <c r="J22" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K22" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
@@ -2057,10 +2063,10 @@
         <v>0</v>
       </c>
       <c r="P22" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q22" s="2">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="R22" s="2">
         <v>0</v>
@@ -2072,85 +2078,93 @@
         <v>-2</v>
       </c>
       <c r="U22" s="2">
-        <v>10</v>
+        <f t="shared" si="0"/>
+        <v>16</v>
       </c>
       <c r="V22" s="2"/>
       <c r="W22" s="2"/>
     </row>
-    <row r="23" spans="1:23" ht="22.5" hidden="1">
+    <row r="23" spans="1:23" ht="78.75">
       <c r="A23" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D23" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K23" s="2">
         <v>7</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
+      <c r="M23" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O23" s="2">
         <v>0</v>
       </c>
       <c r="P23" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q23" s="2">
         <v>7</v>
       </c>
       <c r="R23" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="S23" s="2">
         <v>0</v>
       </c>
       <c r="T23" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="U23" s="2">
-        <v>11</v>
-      </c>
-      <c r="V23" s="2"/>
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="V23" s="2">
+        <v>2</v>
+      </c>
       <c r="W23" s="2"/>
     </row>
-    <row r="24" spans="1:23" ht="90">
+    <row r="24" spans="1:23" ht="22.5">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>100</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J24" s="2">
         <v>8</v>
@@ -2177,45 +2191,42 @@
         <v>0</v>
       </c>
       <c r="T24" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="U24" s="2">
-        <v>10</v>
-      </c>
-      <c r="V24" s="2">
-        <v>2</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="V24" s="2"/>
       <c r="W24" s="2"/>
     </row>
-    <row r="25" spans="1:23" ht="101.25">
+    <row r="25" spans="1:23" ht="45">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E25" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="F25" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I25" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="G25" s="2"/>
+      <c r="H25" s="2"/>
+      <c r="I25" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J25" s="2">
         <v>8</v>
       </c>
       <c r="K25" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2227,52 +2238,51 @@
         <v>8</v>
       </c>
       <c r="Q25" s="2">
+        <v>4</v>
+      </c>
+      <c r="R25" s="2">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2">
+        <v>0</v>
+      </c>
+      <c r="T25" s="2">
+        <v>-2</v>
+      </c>
+      <c r="U25" s="2">
+        <f t="shared" si="0"/>
+        <v>14</v>
+      </c>
+      <c r="V25" s="2"/>
+      <c r="W25" s="2"/>
+    </row>
+    <row r="26" spans="1:23" ht="90">
+      <c r="A26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J26" s="2">
+        <v>8</v>
+      </c>
+      <c r="K26" s="2">
         <v>3</v>
-      </c>
-      <c r="R25" s="2">
-        <v>0</v>
-      </c>
-      <c r="S25" s="2">
-        <v>0</v>
-      </c>
-      <c r="T25" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U25" s="2">
-        <v>10</v>
-      </c>
-      <c r="V25" s="2">
-        <v>2</v>
-      </c>
-      <c r="W25" s="2"/>
-    </row>
-    <row r="26" spans="1:23" ht="45" hidden="1">
-      <c r="A26" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2">
-        <v>4</v>
-      </c>
-      <c r="K26" s="2">
-        <v>7</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -2281,10 +2291,10 @@
         <v>0</v>
       </c>
       <c r="P26" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q26" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R26" s="2">
         <v>0</v>
@@ -2293,60 +2303,61 @@
         <v>0</v>
       </c>
       <c r="T26" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="U26" s="2">
-        <v>9</v>
-      </c>
-      <c r="V26" s="2"/>
+        <f t="shared" si="0"/>
+        <v>13</v>
+      </c>
+      <c r="V26" s="2">
+        <v>2</v>
+      </c>
       <c r="W26" s="2"/>
     </row>
-    <row r="27" spans="1:23" ht="78.75" hidden="1">
+    <row r="27" spans="1:23" ht="101.25">
       <c r="A27" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H27" s="2"/>
+        <v>114</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K27" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L27" s="2"/>
-      <c r="M27" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>127</v>
-      </c>
+      <c r="M27" s="2"/>
+      <c r="N27" s="2"/>
       <c r="O27" s="2">
         <v>0</v>
       </c>
       <c r="P27" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="R27" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2">
         <v>0</v>
@@ -2355,14 +2366,15 @@
         <v>-1</v>
       </c>
       <c r="U27" s="2">
-        <v>9</v>
+        <f t="shared" si="0"/>
+        <v>13</v>
       </c>
       <c r="V27" s="2">
         <v>2</v>
       </c>
       <c r="W27" s="2"/>
     </row>
-    <row r="28" spans="1:23" ht="123.75" hidden="1">
+    <row r="28" spans="1:23" ht="123.75">
       <c r="A28" s="5" t="s">
         <v>24</v>
       </c>
@@ -2370,17 +2382,17 @@
         <v>54</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -2391,13 +2403,13 @@
         <v>1</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="M28" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="O28" s="2">
         <v>0</v>
@@ -2418,6 +2430,7 @@
         <v>-1</v>
       </c>
       <c r="U28" s="2">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="V28" s="2">
@@ -2425,33 +2438,35 @@
       </c>
       <c r="W28" s="2"/>
     </row>
-    <row r="29" spans="1:23" ht="22.5" hidden="1">
+    <row r="29" spans="1:23" ht="45">
       <c r="A29" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>133</v>
+        <v>91</v>
       </c>
       <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="E29" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="F29" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G29" s="2" t="s">
-        <v>117</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I29" s="2"/>
+        <v>114</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J29" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="K29" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2460,10 +2475,10 @@
         <v>0</v>
       </c>
       <c r="P29" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q29" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R29" s="2">
         <v>0</v>
@@ -2472,131 +2487,134 @@
         <v>0</v>
       </c>
       <c r="T29" s="2">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="U29" s="2">
-        <v>5</v>
+        <f t="shared" si="0"/>
+        <v>8</v>
       </c>
       <c r="V29" s="2"/>
       <c r="W29" s="2"/>
     </row>
-    <row r="30" spans="1:23" ht="45">
+    <row r="30" spans="1:23" ht="33.75">
       <c r="A30" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G30" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="H30" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>117</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="I30" s="2"/>
       <c r="J30" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K30" s="2">
-        <v>4</v>
-      </c>
-      <c r="L30" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L30" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2">
         <v>0</v>
       </c>
       <c r="P30" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q30" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R30" s="2">
         <v>0</v>
       </c>
       <c r="S30" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T30" s="2">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="U30" s="2">
-        <v>4</v>
+        <f t="shared" si="0"/>
+        <v>7</v>
       </c>
       <c r="V30" s="2"/>
-      <c r="W30" s="2"/>
-    </row>
-    <row r="31" spans="1:23" ht="33.75" hidden="1">
+      <c r="W30" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" ht="56.25">
       <c r="A31" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2" t="s">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I31" s="2"/>
+        <v>114</v>
+      </c>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J31" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K31" s="2">
-        <v>1</v>
-      </c>
-      <c r="L31" s="2" t="s">
-        <v>123</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L31" s="2"/>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2">
         <v>0</v>
       </c>
       <c r="P31" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q31" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R31" s="2">
         <v>0</v>
       </c>
       <c r="S31" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T31" s="2">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="U31" s="2">
-        <v>7</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="V31" s="2"/>
-      <c r="W31" s="2">
-        <v>5</v>
-      </c>
+      <c r="W31" s="2"/>
     </row>
     <row r="32" spans="1:23" ht="101.25">
       <c r="A32" s="5" t="s">
@@ -2606,23 +2624,23 @@
         <v>57</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G32" s="2"/>
       <c r="H32" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J32" s="2">
         <v>4</v>
@@ -2652,7 +2670,8 @@
         <v>-6</v>
       </c>
       <c r="U32" s="2">
-        <v>2</v>
+        <f t="shared" si="0"/>
+        <v>6</v>
       </c>
       <c r="V32" s="2">
         <v>2</v>
@@ -2663,33 +2682,31 @@
     </row>
     <row r="33" spans="1:23" ht="22.5">
       <c r="A33" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>94</v>
+        <v>129</v>
       </c>
       <c r="D33" s="2"/>
-      <c r="E33" s="2" t="s">
-        <v>132</v>
-      </c>
+      <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2" t="s">
-        <v>117</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I33" s="2"/>
       <c r="J33" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K33" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -2698,10 +2715,10 @@
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q33" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R33" s="2">
         <v>0</v>
@@ -2710,151 +2727,154 @@
         <v>0</v>
       </c>
       <c r="T33" s="2">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="U33" s="2">
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>5</v>
       </c>
       <c r="V33" s="2"/>
       <c r="W33" s="2"/>
     </row>
-    <row r="34" spans="1:23" ht="56.25">
+    <row r="34" spans="1:23" ht="90">
       <c r="A34" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="D34" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="E34" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2" t="s">
-        <v>117</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I34" s="2"/>
       <c r="J34" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K34" s="2">
-        <v>2</v>
-      </c>
-      <c r="L34" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>121</v>
+      </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2">
         <v>0</v>
       </c>
       <c r="P34" s="2">
+        <v>5</v>
+      </c>
+      <c r="Q34" s="2">
+        <v>0</v>
+      </c>
+      <c r="R34" s="2">
+        <v>0</v>
+      </c>
+      <c r="S34" s="2">
+        <v>1</v>
+      </c>
+      <c r="T34" s="2">
+        <v>-1</v>
+      </c>
+      <c r="U34" s="2">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="V34" s="2"/>
+      <c r="W34" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" ht="56.25">
+      <c r="A35" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J35" s="2">
         <v>4</v>
       </c>
-      <c r="Q34" s="2">
+      <c r="K35" s="2">
         <v>2</v>
       </c>
-      <c r="R34" s="2">
-        <v>0</v>
-      </c>
-      <c r="S34" s="2">
-        <v>0</v>
-      </c>
-      <c r="T34" s="2">
-        <v>-3</v>
-      </c>
-      <c r="U34" s="2">
-        <v>3</v>
-      </c>
-      <c r="V34" s="2"/>
-      <c r="W34" s="2"/>
-    </row>
-    <row r="35" spans="1:23" ht="90" hidden="1">
-      <c r="A35" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2">
-        <v>5</v>
-      </c>
-      <c r="K35" s="2">
-        <v>1</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>124</v>
-      </c>
+      <c r="L35" s="2"/>
       <c r="M35" s="2"/>
       <c r="N35" s="2"/>
       <c r="O35" s="2">
         <v>0</v>
       </c>
       <c r="P35" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q35" s="2">
+        <v>2</v>
+      </c>
+      <c r="R35" s="2">
+        <v>0</v>
+      </c>
+      <c r="S35" s="2">
+        <v>0</v>
+      </c>
+      <c r="T35" s="2">
+        <v>-3</v>
+      </c>
+      <c r="U35" s="2">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="Q35" s="2">
-        <v>0</v>
-      </c>
-      <c r="R35" s="2">
-        <v>0</v>
-      </c>
-      <c r="S35" s="2">
-        <v>1</v>
-      </c>
-      <c r="T35" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U35" s="2">
-        <v>5</v>
-      </c>
       <c r="V35" s="2"/>
-      <c r="W35" s="2">
-        <v>2</v>
-      </c>
+      <c r="W35" s="2"/>
     </row>
     <row r="36" spans="1:23" ht="22.5">
       <c r="A36" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>61</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2886,112 +2906,120 @@
         <v>0</v>
       </c>
       <c r="U36" s="2">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="V36" s="2"/>
       <c r="W36" s="2"/>
     </row>
-    <row r="37" spans="1:23" ht="45">
+    <row r="37" spans="1:23" ht="78.75">
       <c r="A37" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2" t="s">
-        <v>109</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E37" s="2"/>
       <c r="F37" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G37" s="2"/>
-      <c r="H37" s="2" t="s">
-        <v>117</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K37" s="2">
         <v>1</v>
       </c>
       <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
+      <c r="M37" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O37" s="2">
         <v>0</v>
       </c>
       <c r="P37" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="2">
+        <v>0</v>
+      </c>
+      <c r="R37" s="2">
         <v>4</v>
       </c>
-      <c r="Q37" s="2">
-        <v>0</v>
-      </c>
-      <c r="R37" s="2">
-        <v>0</v>
-      </c>
       <c r="S37" s="2">
         <v>0</v>
       </c>
       <c r="T37" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="U37" s="2">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="V37" s="2">
         <v>2</v>
       </c>
-      <c r="V37" s="2"/>
       <c r="W37" s="2"/>
     </row>
-    <row r="38" spans="1:23" ht="78.75" hidden="1">
+    <row r="38" spans="1:23" ht="78.75">
       <c r="A38" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K38" s="2">
         <v>1</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2" t="s">
-        <v>125</v>
+        <v>63</v>
       </c>
       <c r="N38" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="O38" s="2">
         <v>0</v>
       </c>
       <c r="P38" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q38" s="2">
         <v>0</v>
       </c>
       <c r="R38" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="S38" s="2">
         <v>0</v>
@@ -3000,6 +3028,7 @@
         <v>-1</v>
       </c>
       <c r="U38" s="2">
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="V38" s="2">
@@ -3007,87 +3036,82 @@
       </c>
       <c r="W38" s="2"/>
     </row>
-    <row r="39" spans="1:23" ht="78.75" hidden="1">
+    <row r="39" spans="1:23" ht="45">
       <c r="A39" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E39" s="2"/>
       <c r="F39" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H39" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="I39" s="2"/>
       <c r="J39" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K39" s="2">
         <v>1</v>
       </c>
       <c r="L39" s="2"/>
-      <c r="M39" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>129</v>
-      </c>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
       <c r="O39" s="2">
         <v>0</v>
       </c>
       <c r="P39" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q39" s="2">
         <v>0</v>
       </c>
       <c r="R39" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S39" s="2">
         <v>0</v>
       </c>
       <c r="T39" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="U39" s="2">
-        <v>3</v>
-      </c>
-      <c r="V39" s="2">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
+      <c r="V39" s="2"/>
       <c r="W39" s="2"/>
     </row>
-    <row r="40" spans="1:23" ht="33.75" hidden="1">
+    <row r="40" spans="1:23" ht="33.75">
       <c r="A40" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2">
@@ -3118,6 +3142,7 @@
         <v>-2</v>
       </c>
       <c r="U40" s="2">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V40" s="2"/>
@@ -3125,27 +3150,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="157.5" hidden="1">
+    <row r="41" spans="1:23" ht="157.5">
       <c r="A41" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -3177,6 +3202,7 @@
         <v>-1</v>
       </c>
       <c r="U41" s="2">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="V41" s="2"/>
@@ -3185,13 +3211,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W41">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Cavalry / Leaper"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:W41"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Value pieces by reach
A piece's direction and speed bonuses give way to its reach: the cells
it could move to or capture on from d4 of an empty 8x8 board. Reach
follows chess's own values, and makes a compound piece worth about its
parts; doubled speed had put long leaps and hops above the Rook.

Bonuses set on the old scale are brought to the new one: the Xiangqi
General's flying-general capture is a power bonus of 7, not a speed;
hoppers are reached with a piece next to them, and the Cannons' hop
bonus goes, the Xiangqi Cannon taking -4 for capturing only by hopping;
binding costs -1 for half the board and -2 for less. The sheet drops
its speed-bonus column, computes each value plainly, and is sorted by
value again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$W$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$41</definedName>
   </definedNames>
   <calcPr calcId="114210" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="134">
   <si>
     <t>Piece Class</t>
   </si>
@@ -416,6 +416,9 @@
   </si>
   <si>
     <t>Must jump over exactly one intervening piece; may neither jump over nor capture a Cannon of either kind.</t>
+  </si>
+  <si>
+    <t>Reach (cells it could reach from d4 on an empty 8×8 board)</t>
   </si>
 </sst>
 </file>
@@ -807,7 +810,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W41"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="6"/>
@@ -815,7 +818,7 @@
     <col min="12" max="12" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="4" customFormat="1" ht="56.25">
+    <row r="1" spans="1:22" s="4" customFormat="1" ht="56.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -862,31 +865,28 @@
         <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="33.75">
+    <row r="2" spans="1:22" ht="33.75">
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
@@ -921,10 +921,10 @@
         <v>60</v>
       </c>
       <c r="P2" s="2">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="Q2" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R2" s="2">
         <v>0</v>
@@ -933,84 +933,76 @@
         <v>0</v>
       </c>
       <c r="T2" s="2">
-        <v>0</v>
-      </c>
-      <c r="U2" s="2">
-        <f t="shared" ref="U2:U41" si="0">O2+P2+Q2*2+R2+S2+T2</f>
-        <v>82</v>
-      </c>
+        <f>O2+P2+Q2+R2+S2</f>
+        <v>78</v>
+      </c>
+      <c r="U2" s="2"/>
       <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-    </row>
-    <row r="3" spans="1:23" ht="33.75">
+    </row>
+    <row r="3" spans="1:22" ht="33.75">
       <c r="A3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="2" t="s">
-        <v>105</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J3" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K3" s="2">
-        <v>7</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>116</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L3" s="2"/>
       <c r="M3" s="2"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2">
         <v>60</v>
       </c>
       <c r="P3" s="2">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="Q3" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R3" s="2">
         <v>0</v>
       </c>
       <c r="S3" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T3" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U3" s="2">
-        <f t="shared" si="0"/>
-        <v>79</v>
-      </c>
+        <f>O3+P3+Q3+R3+S3</f>
+        <v>76</v>
+      </c>
+      <c r="U3" s="2"/>
       <c r="V3" s="2"/>
-      <c r="W3" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" ht="33.75">
+    </row>
+    <row r="4" spans="1:22" ht="22.5">
       <c r="A4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -1023,16 +1015,16 @@
       <c r="H4" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2">
         <v>8</v>
       </c>
       <c r="K4" s="2">
-        <v>3</v>
-      </c>
-      <c r="L4" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>117</v>
+      </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2">
@@ -1042,54 +1034,51 @@
         <v>8</v>
       </c>
       <c r="Q4" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R4" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S4" s="2">
         <v>0</v>
       </c>
       <c r="T4" s="2">
-        <v>0</v>
-      </c>
-      <c r="U4" s="2">
-        <f t="shared" si="0"/>
-        <v>74</v>
-      </c>
+        <f>O4+P4+Q4+R4+S4</f>
+        <v>70</v>
+      </c>
+      <c r="U4" s="2"/>
       <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-    </row>
-    <row r="5" spans="1:23" ht="22.5">
+    </row>
+    <row r="5" spans="1:22" ht="33.75">
       <c r="A5" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="E5" s="2" t="s">
+        <v>105</v>
+      </c>
       <c r="F5" s="2" t="s">
         <v>111</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K5" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1097,28 +1086,27 @@
         <v>60</v>
       </c>
       <c r="P5" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="Q5" s="2">
         <v>0</v>
       </c>
       <c r="R5" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="S5" s="2">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="T5" s="2">
-        <v>0</v>
-      </c>
-      <c r="U5" s="2">
-        <f t="shared" si="0"/>
-        <v>70</v>
-      </c>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-    </row>
-    <row r="6" spans="1:23" ht="78.75">
+        <f>O5+P5+Q5+R5+S5</f>
+        <v>69</v>
+      </c>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="78.75">
       <c r="A6" s="5" t="s">
         <v>23</v>
       </c>
@@ -1160,25 +1148,22 @@
         <v>5</v>
       </c>
       <c r="Q6" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R6" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="S6" s="2">
         <v>0</v>
       </c>
       <c r="T6" s="2">
-        <v>0</v>
-      </c>
-      <c r="U6" s="2">
-        <f t="shared" si="0"/>
+        <f>O6+P6+Q6+R6+S6</f>
         <v>68</v>
       </c>
+      <c r="U6" s="2"/>
       <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-    </row>
-    <row r="7" spans="1:23" ht="33.75">
+    </row>
+    <row r="7" spans="1:22" ht="33.75">
       <c r="A7" s="5" t="s">
         <v>23</v>
       </c>
@@ -1223,24 +1208,21 @@
         <v>0</v>
       </c>
       <c r="R7" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S7" s="2">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="T7" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U7" s="2">
-        <f t="shared" si="0"/>
+        <f>O7+P7+Q7+R7+S7</f>
         <v>68</v>
       </c>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2">
+      <c r="U7" s="2"/>
+      <c r="V7" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:23" ht="33.75">
+    <row r="8" spans="1:22" ht="33.75">
       <c r="A8" s="5" t="s">
         <v>23</v>
       </c>
@@ -1287,16 +1269,13 @@
         <v>0</v>
       </c>
       <c r="T8" s="2">
-        <v>0</v>
-      </c>
-      <c r="U8" s="2">
-        <f t="shared" si="0"/>
+        <f>O8+P8+Q8+R8+S8</f>
         <v>66</v>
       </c>
+      <c r="U8" s="2"/>
       <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-    </row>
-    <row r="9" spans="1:23" ht="33.75">
+    </row>
+    <row r="9" spans="1:22" ht="33.75">
       <c r="A9" s="5" t="s">
         <v>25</v>
       </c>
@@ -1333,54 +1312,51 @@
         <v>0</v>
       </c>
       <c r="P9" s="2">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="Q9" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R9" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S9" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T9" s="2">
-        <v>0</v>
-      </c>
-      <c r="U9" s="2">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
+        <f>O9+P9+Q9+R9+S9</f>
+        <v>37</v>
+      </c>
+      <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-    </row>
-    <row r="10" spans="1:23" ht="157.5">
+    </row>
+    <row r="10" spans="1:22" ht="22.5">
       <c r="A10" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>95</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G10" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I10" s="2"/>
       <c r="J10" s="2">
         <v>8</v>
       </c>
       <c r="K10" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -1389,10 +1365,10 @@
         <v>0</v>
       </c>
       <c r="P10" s="2">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="Q10" s="2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="R10" s="2">
         <v>0</v>
@@ -1401,24 +1377,21 @@
         <v>0</v>
       </c>
       <c r="T10" s="2">
-        <v>0</v>
-      </c>
-      <c r="U10" s="2">
-        <f t="shared" si="0"/>
-        <v>24</v>
-      </c>
+        <f>O10+P10+Q10+R10+S10</f>
+        <v>27</v>
+      </c>
+      <c r="U10" s="2"/>
       <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-    </row>
-    <row r="11" spans="1:23" ht="22.5">
+    </row>
+    <row r="11" spans="1:22" ht="33.75">
       <c r="A11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -1428,10 +1401,10 @@
       <c r="G11" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J11" s="2">
         <v>8</v>
       </c>
@@ -1445,10 +1418,10 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="Q11" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2">
         <v>0</v>
@@ -1457,16 +1430,13 @@
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <v>0</v>
-      </c>
-      <c r="U11" s="2">
-        <f t="shared" si="0"/>
+        <f>O11+P11+Q11+R11+S11</f>
         <v>22</v>
       </c>
+      <c r="U11" s="2"/>
       <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-    </row>
-    <row r="12" spans="1:23" ht="22.5">
+    </row>
+    <row r="12" spans="1:22" ht="22.5">
       <c r="A12" s="5" t="s">
         <v>25</v>
       </c>
@@ -1501,10 +1471,10 @@
         <v>0</v>
       </c>
       <c r="P12" s="2">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="Q12" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R12" s="2">
         <v>0</v>
@@ -1513,34 +1483,31 @@
         <v>0</v>
       </c>
       <c r="T12" s="2">
-        <v>0</v>
-      </c>
-      <c r="U12" s="2">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
+        <f>O12+P12+Q12+R12+S12</f>
+        <v>21</v>
+      </c>
+      <c r="U12" s="2"/>
       <c r="V12" s="2"/>
-      <c r="W12" s="2"/>
-    </row>
-    <row r="13" spans="1:23" ht="33.75">
+    </row>
+    <row r="13" spans="1:22" ht="33.75">
       <c r="A13" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="I13" s="2" t="s">
         <v>114</v>
       </c>
@@ -1557,10 +1524,10 @@
         <v>0</v>
       </c>
       <c r="P13" s="2">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="Q13" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R13" s="2">
         <v>0</v>
@@ -1569,16 +1536,13 @@
         <v>0</v>
       </c>
       <c r="T13" s="2">
-        <v>0</v>
-      </c>
-      <c r="U13" s="2">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
+        <f>O13+P13+Q13+R13+S13</f>
+        <v>21</v>
+      </c>
+      <c r="U13" s="2"/>
       <c r="V13" s="2"/>
-      <c r="W13" s="2"/>
-    </row>
-    <row r="14" spans="1:23" ht="33.75">
+    </row>
+    <row r="14" spans="1:22" ht="33.75">
       <c r="A14" s="5" t="s">
         <v>25</v>
       </c>
@@ -1613,10 +1577,10 @@
         <v>0</v>
       </c>
       <c r="P14" s="2">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="Q14" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R14" s="2">
         <v>0</v>
@@ -1625,39 +1589,34 @@
         <v>0</v>
       </c>
       <c r="T14" s="2">
-        <v>0</v>
-      </c>
-      <c r="U14" s="2">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
+        <f>O14+P14+Q14+R14+S14</f>
+        <v>17</v>
+      </c>
+      <c r="U14" s="2"/>
       <c r="V14" s="2"/>
-      <c r="W14" s="2"/>
-    </row>
-    <row r="15" spans="1:23" ht="33.75">
+    </row>
+    <row r="15" spans="1:22" ht="22.5">
       <c r="A15" s="5" t="s">
         <v>25</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G15" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
       <c r="J15" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K15" s="2">
         <v>7</v>
@@ -1669,10 +1628,10 @@
         <v>0</v>
       </c>
       <c r="P15" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="Q15" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2">
         <v>0</v>
@@ -1681,38 +1640,31 @@
         <v>0</v>
       </c>
       <c r="T15" s="2">
-        <v>0</v>
-      </c>
-      <c r="U15" s="2">
-        <f t="shared" si="0"/>
-        <v>22</v>
-      </c>
+        <f>O15+P15+Q15+R15+S15</f>
+        <v>14</v>
+      </c>
+      <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="2"/>
-    </row>
-    <row r="16" spans="1:23" ht="112.5">
+    </row>
+    <row r="16" spans="1:22" ht="157.5">
       <c r="A16" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
         <v>114</v>
       </c>
@@ -1720,7 +1672,7 @@
         <v>8</v>
       </c>
       <c r="K16" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -1729,10 +1681,10 @@
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="Q16" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2">
         <v>0</v>
@@ -1741,36 +1693,33 @@
         <v>0</v>
       </c>
       <c r="T16" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U16" s="2">
-        <f t="shared" si="0"/>
-        <v>21</v>
-      </c>
-      <c r="V16" s="2">
-        <v>3</v>
-      </c>
-      <c r="W16" s="2"/>
-    </row>
-    <row r="17" spans="1:23" ht="112.5">
+        <f>O16+P16+Q16+R16+S16</f>
+        <v>12</v>
+      </c>
+      <c r="U16" s="2"/>
+      <c r="V16" s="2"/>
+    </row>
+    <row r="17" spans="1:22" ht="45">
       <c r="A17" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="F17" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G17" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H17" s="2"/>
+        <v>111</v>
+      </c>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2">
         <v>4</v>
@@ -1785,51 +1734,44 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="Q17" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R17" s="2">
         <v>0</v>
       </c>
       <c r="S17" s="2">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="T17" s="2">
-        <v>0</v>
-      </c>
-      <c r="U17" s="2">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
+        <f>O17+P17+Q17+R17+S17</f>
+        <v>12</v>
+      </c>
+      <c r="U17" s="2"/>
       <c r="V17" s="2"/>
-      <c r="W17" s="2"/>
-    </row>
-    <row r="18" spans="1:23" ht="101.25">
+    </row>
+    <row r="18" spans="1:22" ht="112.5">
       <c r="A18" s="5" t="s">
         <v>27</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>132</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>114</v>
       </c>
       <c r="H18" s="2"/>
-      <c r="I18" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="I18" s="2"/>
       <c r="J18" s="2">
         <v>4</v>
       </c>
@@ -1843,54 +1785,53 @@
         <v>0</v>
       </c>
       <c r="P18" s="2">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="Q18" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R18" s="2">
         <v>0</v>
       </c>
       <c r="S18" s="2">
-        <v>2</v>
+        <v>-4</v>
       </c>
       <c r="T18" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U18" s="2">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="V18" s="2">
-        <v>3</v>
-      </c>
-      <c r="W18" s="2"/>
-    </row>
-    <row r="19" spans="1:23" ht="22.5">
+        <f>O18+P18+Q18+R18+S18</f>
+        <v>10</v>
+      </c>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+    </row>
+    <row r="19" spans="1:22" ht="101.25">
       <c r="A19" s="5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>132</v>
+      </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G19" s="2"/>
+      <c r="G19" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
         <v>114</v>
       </c>
       <c r="J19" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K19" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -1899,52 +1840,51 @@
         <v>0</v>
       </c>
       <c r="P19" s="2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q19" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R19" s="2">
         <v>0</v>
       </c>
       <c r="S19" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T19" s="2">
-        <v>0</v>
+        <f>O19+P19+Q19+R19+S19</f>
+        <v>8</v>
       </c>
       <c r="U19" s="2">
-        <f t="shared" si="0"/>
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="V19" s="2"/>
-      <c r="W19" s="2"/>
-    </row>
-    <row r="20" spans="1:23" ht="22.5">
+    </row>
+    <row r="20" spans="1:22" ht="45">
       <c r="A20" s="5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G20" s="2"/>
       <c r="H20" s="2"/>
-      <c r="I20" s="2"/>
+      <c r="I20" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J20" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K20" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
@@ -1953,10 +1893,10 @@
         <v>0</v>
       </c>
       <c r="P20" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q20" s="2">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="R20" s="2">
         <v>0</v>
@@ -1965,24 +1905,21 @@
         <v>0</v>
       </c>
       <c r="T20" s="2">
-        <v>0</v>
-      </c>
-      <c r="U20" s="2">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
+        <f>O20+P20+Q20+R20+S20</f>
+        <v>8</v>
+      </c>
+      <c r="U20" s="2"/>
       <c r="V20" s="2"/>
-      <c r="W20" s="2"/>
-    </row>
-    <row r="21" spans="1:23" ht="45">
+    </row>
+    <row r="21" spans="1:22" ht="22.5">
       <c r="A21" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -1998,7 +1935,7 @@
         <v>8</v>
       </c>
       <c r="K21" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -2010,7 +1947,7 @@
         <v>8</v>
       </c>
       <c r="Q21" s="2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R21" s="2">
         <v>0</v>
@@ -2019,83 +1956,85 @@
         <v>0</v>
       </c>
       <c r="T21" s="2">
-        <v>0</v>
-      </c>
-      <c r="U21" s="2">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
+        <f>O21+P21+Q21+R21+S21</f>
+        <v>8</v>
+      </c>
+      <c r="U21" s="2"/>
       <c r="V21" s="2"/>
-      <c r="W21" s="2"/>
-    </row>
-    <row r="22" spans="1:23" ht="45">
+    </row>
+    <row r="22" spans="1:22" ht="123.75">
       <c r="A22" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2" t="s">
-        <v>106</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2" t="s">
-        <v>114</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H22" s="2"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K22" s="2">
-        <v>7</v>
-      </c>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L22" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>125</v>
+      </c>
       <c r="O22" s="2">
         <v>0</v>
       </c>
       <c r="P22" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q22" s="2">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="R22" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S22" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T22" s="2">
-        <v>-2</v>
+        <f>O22+P22+Q22+R22+S22</f>
+        <v>8</v>
       </c>
       <c r="U22" s="2">
-        <f t="shared" si="0"/>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="V22" s="2"/>
-      <c r="W22" s="2"/>
-    </row>
-    <row r="23" spans="1:23" ht="78.75">
+    </row>
+    <row r="23" spans="1:22" ht="112.5">
       <c r="A23" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
@@ -2104,60 +2043,59 @@
       <c r="G23" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H23" s="2"/>
-      <c r="I23" s="2"/>
+      <c r="H23" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J23" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K23" s="2">
         <v>7</v>
       </c>
       <c r="L23" s="2"/>
-      <c r="M23" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="N23" s="2" t="s">
-        <v>124</v>
-      </c>
+      <c r="M23" s="2"/>
+      <c r="N23" s="2"/>
       <c r="O23" s="2">
         <v>0</v>
       </c>
       <c r="P23" s="2">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q23" s="2">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2">
+        <v>-1</v>
+      </c>
+      <c r="T23" s="2">
+        <f>O23+P23+Q23+R23+S23</f>
         <v>7</v>
       </c>
-      <c r="R23" s="2">
+      <c r="U23" s="2">
         <v>3</v>
       </c>
-      <c r="S23" s="2">
-        <v>0</v>
-      </c>
-      <c r="T23" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U23" s="2">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="V23" s="2">
-        <v>2</v>
-      </c>
-      <c r="W23" s="2"/>
-    </row>
-    <row r="24" spans="1:23" ht="22.5">
+      <c r="V23" s="2"/>
+    </row>
+    <row r="24" spans="1:22" ht="45">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="E24" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="F24" s="2" t="s">
         <v>111</v>
       </c>
@@ -2170,7 +2108,7 @@
         <v>8</v>
       </c>
       <c r="K24" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
@@ -2182,38 +2120,35 @@
         <v>8</v>
       </c>
       <c r="Q24" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R24" s="2">
         <v>0</v>
       </c>
       <c r="S24" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T24" s="2">
-        <v>0</v>
-      </c>
-      <c r="U24" s="2">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
+        <f>O24+P24+Q24+R24+S24</f>
+        <v>7</v>
+      </c>
+      <c r="U24" s="2"/>
       <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
-    </row>
-    <row r="25" spans="1:23" ht="45">
+    </row>
+    <row r="25" spans="1:22" ht="90">
       <c r="A25" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2" t="s">
-        <v>106</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
         <v>111</v>
       </c>
@@ -2226,7 +2161,7 @@
         <v>8</v>
       </c>
       <c r="K25" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2238,46 +2173,47 @@
         <v>8</v>
       </c>
       <c r="Q25" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R25" s="2">
         <v>0</v>
       </c>
       <c r="S25" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T25" s="2">
-        <v>-2</v>
+        <f>O25+P25+Q25+R25+S25</f>
+        <v>7</v>
       </c>
       <c r="U25" s="2">
-        <f t="shared" si="0"/>
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="V25" s="2"/>
-      <c r="W25" s="2"/>
-    </row>
-    <row r="26" spans="1:23" ht="90">
+    </row>
+    <row r="26" spans="1:22" ht="101.25">
       <c r="A26" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2"/>
-      <c r="I26" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I26" s="2"/>
       <c r="J26" s="2">
         <v>8</v>
       </c>
@@ -2294,40 +2230,37 @@
         <v>8</v>
       </c>
       <c r="Q26" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R26" s="2">
         <v>0</v>
       </c>
       <c r="S26" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T26" s="2">
-        <v>-1</v>
+        <f>O26+P26+Q26+R26+S26</f>
+        <v>7</v>
       </c>
       <c r="U26" s="2">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="V26" s="2">
         <v>2</v>
       </c>
-      <c r="W26" s="2"/>
-    </row>
-    <row r="27" spans="1:23" ht="101.25">
+      <c r="V26" s="2"/>
+    </row>
+    <row r="27" spans="1:22" ht="33.75">
       <c r="A27" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E27" s="2"/>
+        <v>73</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2" t="s">
+        <v>105</v>
+      </c>
       <c r="F27" s="2" t="s">
         <v>111</v>
       </c>
@@ -2342,9 +2275,11 @@
         <v>8</v>
       </c>
       <c r="K27" s="2">
-        <v>3</v>
-      </c>
-      <c r="L27" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="L27" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2">
@@ -2354,42 +2289,39 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R27" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S27" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T27" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U27" s="2">
-        <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
+        <f>O27+P27+Q27+R27+S27</f>
+        <v>7</v>
+      </c>
+      <c r="U27" s="2"/>
       <c r="V27" s="2">
-        <v>2</v>
-      </c>
-      <c r="W27" s="2"/>
-    </row>
-    <row r="28" spans="1:23" ht="123.75">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" ht="78.75">
       <c r="A28" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>114</v>
@@ -2397,76 +2329,69 @@
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
       <c r="J28" s="2">
+        <v>1</v>
+      </c>
+      <c r="K28" s="2">
+        <v>7</v>
+      </c>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="O28" s="2">
+        <v>0</v>
+      </c>
+      <c r="P28" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q28" s="2">
         <v>3</v>
       </c>
-      <c r="K28" s="2">
+      <c r="R28" s="2">
+        <v>0</v>
+      </c>
+      <c r="S28" s="2">
+        <v>-1</v>
+      </c>
+      <c r="T28" s="2">
+        <f>O28+P28+Q28+R28+S28</f>
+        <v>6</v>
+      </c>
+      <c r="U28" s="2">
+        <v>2</v>
+      </c>
+      <c r="V28" s="2"/>
+    </row>
+    <row r="29" spans="1:22" ht="22.5">
+      <c r="A29" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2">
+        <v>5</v>
+      </c>
+      <c r="K29" s="2">
         <v>1</v>
-      </c>
-      <c r="L28" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="O28" s="2">
-        <v>0</v>
-      </c>
-      <c r="P28" s="2">
-        <v>3</v>
-      </c>
-      <c r="Q28" s="2">
-        <v>0</v>
-      </c>
-      <c r="R28" s="2">
-        <v>5</v>
-      </c>
-      <c r="S28" s="2">
-        <v>1</v>
-      </c>
-      <c r="T28" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U28" s="2">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="V28" s="2">
-        <v>2</v>
-      </c>
-      <c r="W28" s="2"/>
-    </row>
-    <row r="29" spans="1:23" ht="45">
-      <c r="A29" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="J29" s="2">
-        <v>4</v>
-      </c>
-      <c r="K29" s="2">
-        <v>4</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2475,10 +2400,10 @@
         <v>0</v>
       </c>
       <c r="P29" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q29" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R29" s="2">
         <v>0</v>
@@ -2487,28 +2412,27 @@
         <v>0</v>
       </c>
       <c r="T29" s="2">
-        <v>-4</v>
-      </c>
-      <c r="U29" s="2">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
+        <f>O29+P29+Q29+R29+S29</f>
+        <v>5</v>
+      </c>
+      <c r="U29" s="2"/>
       <c r="V29" s="2"/>
-      <c r="W29" s="2"/>
-    </row>
-    <row r="30" spans="1:23" ht="33.75">
+    </row>
+    <row r="30" spans="1:22" ht="90">
       <c r="A30" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="E30" s="2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>111</v>
@@ -2517,17 +2441,17 @@
         <v>114</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K30" s="2">
         <v>1</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
@@ -2535,58 +2459,51 @@
         <v>0</v>
       </c>
       <c r="P30" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="Q30" s="2">
         <v>0</v>
       </c>
       <c r="R30" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S30" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T30" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U30" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="V30" s="2"/>
-      <c r="W30" s="2">
+        <f>O30+P30+Q30+R30+S30</f>
         <v>5</v>
       </c>
-    </row>
-    <row r="31" spans="1:23" ht="56.25">
+      <c r="U30" s="2"/>
+      <c r="V30" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" ht="22.5">
       <c r="A31" s="5" t="s">
         <v>26</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="D31" s="2"/>
-      <c r="E31" s="2" t="s">
-        <v>128</v>
-      </c>
+      <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G31" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2" t="s">
         <v>114</v>
       </c>
       <c r="J31" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K31" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -2598,7 +2515,7 @@
         <v>4</v>
       </c>
       <c r="Q31" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R31" s="2">
         <v>0</v>
@@ -2607,46 +2524,37 @@
         <v>0</v>
       </c>
       <c r="T31" s="2">
-        <v>-4</v>
-      </c>
-      <c r="U31" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
+        <f>O31+P31+Q31+R31+S31</f>
+        <v>4</v>
+      </c>
+      <c r="U31" s="2"/>
       <c r="V31" s="2"/>
-      <c r="W31" s="2"/>
-    </row>
-    <row r="32" spans="1:23" ht="101.25">
+    </row>
+    <row r="32" spans="1:22" ht="22.5">
       <c r="A32" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>107</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G32" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
       <c r="J32" s="2">
         <v>4</v>
       </c>
       <c r="K32" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
@@ -2658,39 +2566,34 @@
         <v>4</v>
       </c>
       <c r="Q32" s="2">
+        <v>0</v>
+      </c>
+      <c r="R32" s="2">
+        <v>0</v>
+      </c>
+      <c r="S32" s="2">
+        <v>0</v>
+      </c>
+      <c r="T32" s="2">
+        <f>O32+P32+Q32+R32+S32</f>
         <v>4</v>
       </c>
-      <c r="R32" s="2">
-        <v>0</v>
-      </c>
-      <c r="S32" s="2">
-        <v>0</v>
-      </c>
-      <c r="T32" s="2">
-        <v>-6</v>
-      </c>
-      <c r="U32" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
-      </c>
-      <c r="V32" s="2">
-        <v>2</v>
-      </c>
-      <c r="W32" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:23" ht="22.5">
+      <c r="U32" s="2"/>
+      <c r="V32" s="2"/>
+    </row>
+    <row r="33" spans="1:22" ht="78.75">
       <c r="A33" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="D33" s="2"/>
+        <v>90</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
         <v>111</v>
@@ -2698,137 +2601,131 @@
       <c r="G33" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H33" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K33" s="2">
         <v>1</v>
       </c>
       <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
+      <c r="M33" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O33" s="2">
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="Q33" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R33" s="2">
         <v>0</v>
       </c>
       <c r="S33" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T33" s="2">
-        <v>0</v>
+        <f>O33+P33+Q33+R33+S33</f>
+        <v>4</v>
       </c>
       <c r="U33" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V33" s="2"/>
-      <c r="W33" s="2"/>
-    </row>
-    <row r="34" spans="1:23" ht="90">
+    </row>
+    <row r="34" spans="1:22" ht="78.75">
       <c r="A34" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>130</v>
+        <v>90</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>109</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H34" s="2" t="s">
-        <v>115</v>
-      </c>
+      <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K34" s="2">
         <v>1</v>
       </c>
-      <c r="L34" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>126</v>
+      </c>
       <c r="O34" s="2">
         <v>0</v>
       </c>
       <c r="P34" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Q34" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R34" s="2">
         <v>0</v>
       </c>
       <c r="S34" s="2">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="T34" s="2">
-        <v>-1</v>
+        <f>O34+P34+Q34+R34+S34</f>
+        <v>3</v>
       </c>
       <c r="U34" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="V34" s="2"/>
-      <c r="W34" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:23" ht="56.25">
+    </row>
+    <row r="35" spans="1:22" ht="45">
       <c r="A35" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G35" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2" t="s">
-        <v>114</v>
-      </c>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I35" s="2"/>
       <c r="J35" s="2">
         <v>4</v>
       </c>
       <c r="K35" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
@@ -2840,49 +2737,50 @@
         <v>4</v>
       </c>
       <c r="Q35" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R35" s="2">
         <v>0</v>
       </c>
       <c r="S35" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T35" s="2">
-        <v>-3</v>
-      </c>
-      <c r="U35" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
+        <f>O35+P35+Q35+R35+S35</f>
+        <v>3</v>
+      </c>
+      <c r="U35" s="2"/>
       <c r="V35" s="2"/>
-      <c r="W35" s="2"/>
-    </row>
-    <row r="36" spans="1:23" ht="22.5">
+    </row>
+    <row r="36" spans="1:22" ht="45">
       <c r="A36" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
       <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="E36" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="F36" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J36" s="2">
         <v>4</v>
       </c>
       <c r="K36" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
@@ -2900,169 +2798,160 @@
         <v>0</v>
       </c>
       <c r="S36" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T36" s="2">
-        <v>0</v>
-      </c>
-      <c r="U36" s="2">
-        <f t="shared" si="0"/>
+        <f>O36+P36+Q36+R36+S36</f>
+        <v>2</v>
+      </c>
+      <c r="U36" s="2"/>
+      <c r="V36" s="2"/>
+    </row>
+    <row r="37" spans="1:22" ht="56.25">
+      <c r="A37" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J37" s="2">
         <v>4</v>
       </c>
-      <c r="V36" s="2"/>
-      <c r="W36" s="2"/>
-    </row>
-    <row r="37" spans="1:23" ht="78.75">
-      <c r="A37" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2">
-        <v>1</v>
-      </c>
       <c r="K37" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L37" s="2"/>
-      <c r="M37" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>124</v>
-      </c>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
       <c r="O37" s="2">
         <v>0</v>
       </c>
       <c r="P37" s="2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q37" s="2">
         <v>0</v>
       </c>
       <c r="R37" s="2">
+        <v>0</v>
+      </c>
+      <c r="S37" s="2">
+        <v>-2</v>
+      </c>
+      <c r="T37" s="2">
+        <f>O37+P37+Q37+R37+S37</f>
+        <v>2</v>
+      </c>
+      <c r="U37" s="2"/>
+      <c r="V37" s="2"/>
+    </row>
+    <row r="38" spans="1:22" ht="101.25">
+      <c r="A38" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G38" s="2"/>
+      <c r="H38" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J38" s="2">
         <v>4</v>
       </c>
-      <c r="S37" s="2">
-        <v>0</v>
-      </c>
-      <c r="T37" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U37" s="2">
-        <f t="shared" si="0"/>
+      <c r="K38" s="2">
+        <v>4</v>
+      </c>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2">
+        <v>0</v>
+      </c>
+      <c r="P38" s="2">
+        <v>4</v>
+      </c>
+      <c r="Q38" s="2">
+        <v>0</v>
+      </c>
+      <c r="R38" s="2">
+        <v>0</v>
+      </c>
+      <c r="S38" s="2">
+        <v>-2</v>
+      </c>
+      <c r="T38" s="2">
+        <f>O38+P38+Q38+R38+S38</f>
+        <v>2</v>
+      </c>
+      <c r="U38" s="2">
+        <v>2</v>
+      </c>
+      <c r="V38" s="2">
         <v>3</v>
       </c>
-      <c r="V37" s="2">
-        <v>2</v>
-      </c>
-      <c r="W37" s="2"/>
-    </row>
-    <row r="38" spans="1:23" ht="78.75">
-      <c r="A38" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="H38" s="2"/>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2">
-        <v>3</v>
-      </c>
-      <c r="K38" s="2">
-        <v>1</v>
-      </c>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N38" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="O38" s="2">
-        <v>0</v>
-      </c>
-      <c r="P38" s="2">
-        <v>3</v>
-      </c>
-      <c r="Q38" s="2">
-        <v>0</v>
-      </c>
-      <c r="R38" s="2">
-        <v>1</v>
-      </c>
-      <c r="S38" s="2">
-        <v>0</v>
-      </c>
-      <c r="T38" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U38" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="V38" s="2">
-        <v>2</v>
-      </c>
-      <c r="W38" s="2"/>
-    </row>
-    <row r="39" spans="1:23" ht="45">
+    </row>
+    <row r="39" spans="1:22" ht="56.25">
       <c r="A39" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G39" s="2"/>
-      <c r="H39" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I39" s="2"/>
+      <c r="G39" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="J39" s="2">
         <v>4</v>
       </c>
       <c r="K39" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
@@ -3080,19 +2969,16 @@
         <v>0</v>
       </c>
       <c r="S39" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T39" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U39" s="2">
-        <f t="shared" si="0"/>
+        <f>O39+P39+Q39+R39+S39</f>
         <v>2</v>
       </c>
+      <c r="U39" s="2"/>
       <c r="V39" s="2"/>
-      <c r="W39" s="2"/>
-    </row>
-    <row r="40" spans="1:23" ht="33.75">
+    </row>
+    <row r="40" spans="1:22" ht="33.75">
       <c r="A40" s="5" t="s">
         <v>24</v>
       </c>
@@ -3136,21 +3022,18 @@
         <v>0</v>
       </c>
       <c r="S40" s="2">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="T40" s="2">
-        <v>-2</v>
-      </c>
-      <c r="U40" s="2">
-        <f t="shared" si="0"/>
+        <f>O40+P40+Q40+R40+S40</f>
         <v>2</v>
       </c>
-      <c r="V40" s="2"/>
-      <c r="W40" s="2">
+      <c r="U40" s="2"/>
+      <c r="V40" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:23" ht="157.5">
+    <row r="41" spans="1:22" ht="157.5">
       <c r="A41" s="5" t="s">
         <v>24</v>
       </c>
@@ -3196,22 +3079,19 @@
         <v>0</v>
       </c>
       <c r="S41" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T41" s="2">
-        <v>-1</v>
-      </c>
-      <c r="U41" s="2">
-        <f t="shared" si="0"/>
+        <f>O41+P41+Q41+R41+S41</f>
         <v>2</v>
       </c>
-      <c r="V41" s="2"/>
-      <c r="W41" s="2">
+      <c r="U41" s="2"/>
+      <c r="V41" s="2">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:W41"/>
+  <autoFilter ref="A1:V41"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Price the lifts that were missing, and propose pricing promotions
The Knightrider's movement restriction lifts for 3, each Soldier's for
2; the other lift prices stay as they were. A promotion is priced as
an option: the gain it brings over the distance to reach it, which
shows that a Shogi Pawn or Lance, promoting free into a Gold General
that is now a leader, would be worth more than a Rook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -12,12 +12,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$41</definedName>
   </definedNames>
-  <calcPr calcId="114210" fullCalcOnLoad="1"/>
+  <calcPr calcId="114210"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="131">
   <si>
     <t>Piece Class</t>
   </si>
@@ -64,12 +64,6 @@
     <t>Leader bonus</t>
   </si>
   <si>
-    <t>Direction bonus</t>
-  </si>
-  <si>
-    <t>Speed bonus</t>
-  </si>
-  <si>
     <t>Promotion bonus</t>
   </si>
   <si>
@@ -410,9 +404,6 @@
   </si>
   <si>
     <t>Moves one square forward or sideways; in a palace, also diagonally forward along marked palace lines.</t>
-  </si>
-  <si>
-    <t>Must jump over exactly one intervening piece; cannot jump over a Cannon of either kind.</t>
   </si>
   <si>
     <t>Must jump over exactly one intervening piece; may neither jump over nor capture a Cannon of either kind.</t>
@@ -810,6 +801,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -818,7 +810,7 @@
     <col min="12" max="12" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="4" customFormat="1" ht="56.25">
+    <row r="1" spans="1:22" s="4" customFormat="1" ht="67.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -865,47 +857,47 @@
         <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="Q1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="S1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="U1" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="3" t="s">
+      <c r="V1" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="U1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:22" ht="33.75" hidden="1">
+      <c r="A2" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="V1" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:22" ht="33.75">
-      <c r="A2" s="5" t="s">
-        <v>23</v>
-      </c>
       <c r="B2" s="5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2">
@@ -933,35 +925,35 @@
         <v>0</v>
       </c>
       <c r="T2" s="2">
-        <f>O2+P2+Q2+R2+S2</f>
+        <f t="shared" ref="T2:T41" si="0">O2+P2+Q2+R2+S2</f>
         <v>78</v>
       </c>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
     </row>
-    <row r="3" spans="1:22" ht="33.75">
+    <row r="3" spans="1:22" ht="33.75" hidden="1">
       <c r="A3" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J3" s="2">
         <v>8</v>
@@ -988,32 +980,32 @@
         <v>0</v>
       </c>
       <c r="T3" s="2">
-        <f>O3+P3+Q3+R3+S3</f>
+        <f t="shared" si="0"/>
         <v>76</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
     </row>
-    <row r="4" spans="1:22" ht="22.5">
+    <row r="4" spans="1:22" ht="22.5" hidden="1">
       <c r="A4" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
@@ -1023,7 +1015,7 @@
         <v>1</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -1043,31 +1035,31 @@
         <v>0</v>
       </c>
       <c r="T4" s="2">
-        <f>O4+P4+Q4+R4+S4</f>
+        <f t="shared" si="0"/>
         <v>70</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
     </row>
-    <row r="5" spans="1:22" ht="33.75">
+    <row r="5" spans="1:22" ht="33.75" hidden="1">
       <c r="A5" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1078,7 +1070,7 @@
         <v>7</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1098,7 +1090,7 @@
         <v>-2</v>
       </c>
       <c r="T5" s="2">
-        <f>O5+P5+Q5+R5+S5</f>
+        <f t="shared" si="0"/>
         <v>69</v>
       </c>
       <c r="U5" s="2"/>
@@ -1106,26 +1098,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="78.75">
+    <row r="6" spans="1:22" ht="78.75" hidden="1">
       <c r="A6" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
@@ -1136,10 +1128,10 @@
       </c>
       <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N6" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="O6" s="2">
         <v>60</v>
@@ -1157,34 +1149,34 @@
         <v>0</v>
       </c>
       <c r="T6" s="2">
-        <f>O6+P6+Q6+R6+S6</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
     </row>
-    <row r="7" spans="1:22" ht="33.75">
+    <row r="7" spans="1:22" ht="33.75" hidden="1">
       <c r="A7" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
@@ -1194,7 +1186,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
@@ -1214,7 +1206,7 @@
         <v>-2</v>
       </c>
       <c r="T7" s="2">
-        <f>O7+P7+Q7+R7+S7</f>
+        <f t="shared" si="0"/>
         <v>68</v>
       </c>
       <c r="U7" s="2"/>
@@ -1222,26 +1214,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:22" ht="33.75">
+    <row r="8" spans="1:22" ht="33.75" hidden="1">
       <c r="A8" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
@@ -1269,35 +1261,35 @@
         <v>0</v>
       </c>
       <c r="T8" s="2">
-        <f>O8+P8+Q8+R8+S8</f>
+        <f t="shared" si="0"/>
         <v>66</v>
       </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
     </row>
-    <row r="9" spans="1:22" ht="33.75">
+    <row r="9" spans="1:22" ht="33.75" hidden="1">
       <c r="A9" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J9" s="2">
         <v>8</v>
@@ -1324,32 +1316,32 @@
         <v>0</v>
       </c>
       <c r="T9" s="2">
-        <f>O9+P9+Q9+R9+S9</f>
+        <f t="shared" si="0"/>
         <v>37</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
     </row>
-    <row r="10" spans="1:22" ht="22.5">
+    <row r="10" spans="1:22" ht="22.5" hidden="1">
       <c r="A10" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2">
@@ -1377,33 +1369,33 @@
         <v>0</v>
       </c>
       <c r="T10" s="2">
-        <f>O10+P10+Q10+R10+S10</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:22" ht="33.75">
+    <row r="11" spans="1:22" ht="33.75" hidden="1">
       <c r="A11" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J11" s="2">
         <v>8</v>
@@ -1430,33 +1422,33 @@
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <f>O11+P11+Q11+R11+S11</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:22" ht="22.5">
+    <row r="12" spans="1:22" ht="22.5" hidden="1">
       <c r="A12" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J12" s="2">
         <v>8</v>
@@ -1483,33 +1475,33 @@
         <v>0</v>
       </c>
       <c r="T12" s="2">
-        <f>O12+P12+Q12+R12+S12</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:22" ht="33.75">
+    <row r="13" spans="1:22" ht="33.75" hidden="1">
       <c r="A13" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J13" s="2">
         <v>8</v>
@@ -1536,32 +1528,32 @@
         <v>0</v>
       </c>
       <c r="T13" s="2">
-        <f>O13+P13+Q13+R13+S13</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:22" ht="33.75">
+    <row r="14" spans="1:22" ht="33.75" hidden="1">
       <c r="A14" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2">
@@ -1589,29 +1581,29 @@
         <v>0</v>
       </c>
       <c r="T14" s="2">
-        <f>O14+P14+Q14+R14+S14</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" ht="22.5">
+    <row r="15" spans="1:22" ht="22.5" hidden="1">
       <c r="A15" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -1640,7 +1632,7 @@
         <v>0</v>
       </c>
       <c r="T15" s="2">
-        <f>O15+P15+Q15+R15+S15</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="U15" s="2"/>
@@ -1648,25 +1640,25 @@
     </row>
     <row r="16" spans="1:22" ht="157.5">
       <c r="A16" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J16" s="2">
         <v>8</v>
@@ -1693,32 +1685,34 @@
         <v>0</v>
       </c>
       <c r="T16" s="2">
-        <f>O16+P16+Q16+R16+S16</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="U16" s="2"/>
+      <c r="U16" s="2">
+        <v>3</v>
+      </c>
       <c r="V16" s="2"/>
     </row>
-    <row r="17" spans="1:22" ht="45">
+    <row r="17" spans="1:22" ht="45" hidden="1">
       <c r="A17" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2">
@@ -1746,29 +1740,29 @@
         <v>-1</v>
       </c>
       <c r="T17" s="2">
-        <f>O17+P17+Q17+R17+S17</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:22" ht="112.5">
+    <row r="18" spans="1:22" ht="112.5" hidden="1">
       <c r="A18" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -1797,35 +1791,35 @@
         <v>-4</v>
       </c>
       <c r="T18" s="2">
-        <f>O18+P18+Q18+R18+S18</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:22" ht="101.25">
+    <row r="19" spans="1:22" ht="112.5" hidden="1">
       <c r="A19" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J19" s="2">
         <v>4</v>
@@ -1852,7 +1846,7 @@
         <v>-2</v>
       </c>
       <c r="T19" s="2">
-        <f>O19+P19+Q19+R19+S19</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="U19" s="2">
@@ -1860,25 +1854,25 @@
       </c>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:22" ht="45">
+    <row r="20" spans="1:22" ht="22.5">
       <c r="A20" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J20" s="2">
         <v>8</v>
@@ -1905,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="2">
-        <f>O20+P20+Q20+R20+S20</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="U20" s="2"/>
@@ -1913,23 +1907,23 @@
     </row>
     <row r="21" spans="1:22" ht="22.5">
       <c r="A21" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J21" s="2">
         <v>8</v>
@@ -1956,31 +1950,31 @@
         <v>0</v>
       </c>
       <c r="T21" s="2">
-        <f>O21+P21+Q21+R21+S21</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:22" ht="123.75">
+    <row r="22" spans="1:22" ht="123.75" hidden="1">
       <c r="A22" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -1991,13 +1985,13 @@
         <v>1</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="M22" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="N22" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="O22" s="2">
         <v>0</v>
@@ -2015,7 +2009,7 @@
         <v>-1</v>
       </c>
       <c r="T22" s="2">
-        <f>O22+P22+Q22+R22+S22</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="U22" s="2">
@@ -2023,31 +2017,31 @@
       </c>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:22" ht="112.5">
+    <row r="23" spans="1:22" ht="112.5" hidden="1">
       <c r="A23" s="5" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J23" s="2">
         <v>8</v>
@@ -2074,7 +2068,7 @@
         <v>-1</v>
       </c>
       <c r="T23" s="2">
-        <f>O23+P23+Q23+R23+S23</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U23" s="2">
@@ -2084,25 +2078,25 @@
     </row>
     <row r="24" spans="1:22" ht="45">
       <c r="A24" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J24" s="2">
         <v>8</v>
@@ -2129,7 +2123,7 @@
         <v>-1</v>
       </c>
       <c r="T24" s="2">
-        <f>O24+P24+Q24+R24+S24</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U24" s="2"/>
@@ -2137,25 +2131,25 @@
     </row>
     <row r="25" spans="1:22" ht="90">
       <c r="A25" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J25" s="2">
         <v>8</v>
@@ -2182,7 +2176,7 @@
         <v>-1</v>
       </c>
       <c r="T25" s="2">
-        <f>O25+P25+Q25+R25+S25</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U25" s="2">
@@ -2192,26 +2186,26 @@
     </row>
     <row r="26" spans="1:22" ht="101.25">
       <c r="A26" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I26" s="2"/>
       <c r="J26" s="2">
@@ -2239,7 +2233,7 @@
         <v>-1</v>
       </c>
       <c r="T26" s="2">
-        <f>O26+P26+Q26+R26+S26</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U26" s="2">
@@ -2247,28 +2241,28 @@
       </c>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:22" ht="33.75">
+    <row r="27" spans="1:22" ht="33.75" hidden="1">
       <c r="A27" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I27" s="2"/>
       <c r="J27" s="2">
@@ -2278,7 +2272,7 @@
         <v>1</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
@@ -2298,7 +2292,7 @@
         <v>-2</v>
       </c>
       <c r="T27" s="2">
-        <f>O27+P27+Q27+R27+S27</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="U27" s="2"/>
@@ -2306,25 +2300,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:22" ht="78.75">
+    <row r="28" spans="1:22" ht="78.75" hidden="1">
       <c r="A28" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H28" s="2"/>
       <c r="I28" s="2"/>
@@ -2336,10 +2330,10 @@
       </c>
       <c r="L28" s="2"/>
       <c r="M28" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N28" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="O28" s="2">
         <v>0</v>
@@ -2357,7 +2351,7 @@
         <v>-1</v>
       </c>
       <c r="T28" s="2">
-        <f>O28+P28+Q28+R28+S28</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="U28" s="2">
@@ -2365,26 +2359,26 @@
       </c>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:22" ht="22.5">
+    <row r="29" spans="1:22" ht="22.5" hidden="1">
       <c r="A29" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2">
@@ -2412,36 +2406,36 @@
         <v>0</v>
       </c>
       <c r="T29" s="2">
-        <f>O29+P29+Q29+R29+S29</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="U29" s="2"/>
       <c r="V29" s="2"/>
     </row>
-    <row r="30" spans="1:22" ht="90">
+    <row r="30" spans="1:22" ht="90" hidden="1">
       <c r="A30" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2">
@@ -2451,7 +2445,7 @@
         <v>1</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
@@ -2471,33 +2465,35 @@
         <v>-1</v>
       </c>
       <c r="T30" s="2">
-        <f>O30+P30+Q30+R30+S30</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="U30" s="2"/>
+      <c r="U30" s="2">
+        <v>2</v>
+      </c>
       <c r="V30" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="22.5">
       <c r="A31" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J31" s="2">
         <v>8</v>
@@ -2524,29 +2520,29 @@
         <v>0</v>
       </c>
       <c r="T31" s="2">
-        <f>O31+P31+Q31+R31+S31</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
     </row>
-    <row r="32" spans="1:22" ht="22.5">
+    <row r="32" spans="1:22" hidden="1">
       <c r="A32" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2575,31 +2571,31 @@
         <v>0</v>
       </c>
       <c r="T32" s="2">
-        <f>O32+P32+Q32+R32+S32</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:22" ht="78.75">
+    <row r="33" spans="1:22" ht="78.75" hidden="1">
       <c r="A33" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -2611,10 +2607,10 @@
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N33" s="2" t="s">
         <v>122</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="O33" s="2">
         <v>0</v>
@@ -2632,7 +2628,7 @@
         <v>-1</v>
       </c>
       <c r="T33" s="2">
-        <f>O33+P33+Q33+R33+S33</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="U33" s="2">
@@ -2640,25 +2636,25 @@
       </c>
       <c r="V33" s="2"/>
     </row>
-    <row r="34" spans="1:22" ht="78.75">
+    <row r="34" spans="1:22" ht="78.75" hidden="1">
       <c r="A34" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -2670,10 +2666,10 @@
       </c>
       <c r="L34" s="2"/>
       <c r="M34" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="O34" s="2">
         <v>0</v>
@@ -2691,7 +2687,7 @@
         <v>-1</v>
       </c>
       <c r="T34" s="2">
-        <f>O34+P34+Q34+R34+S34</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="U34" s="2">
@@ -2699,26 +2695,26 @@
       </c>
       <c r="V34" s="2"/>
     </row>
-    <row r="35" spans="1:22" ht="45">
+    <row r="35" spans="1:22" ht="45" hidden="1">
       <c r="A35" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2">
@@ -2746,7 +2742,7 @@
         <v>-1</v>
       </c>
       <c r="T35" s="2">
-        <f>O35+P35+Q35+R35+S35</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="U35" s="2"/>
@@ -2754,27 +2750,27 @@
     </row>
     <row r="36" spans="1:22" ht="45">
       <c r="A36" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J36" s="2">
         <v>4</v>
@@ -2801,7 +2797,7 @@
         <v>-2</v>
       </c>
       <c r="T36" s="2">
-        <f>O36+P36+Q36+R36+S36</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U36" s="2"/>
@@ -2809,27 +2805,27 @@
     </row>
     <row r="37" spans="1:22" ht="56.25">
       <c r="A37" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J37" s="2">
         <v>4</v>
@@ -2856,7 +2852,7 @@
         <v>-2</v>
       </c>
       <c r="T37" s="2">
-        <f>O37+P37+Q37+R37+S37</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U37" s="2"/>
@@ -2864,29 +2860,29 @@
     </row>
     <row r="38" spans="1:22" ht="101.25">
       <c r="A38" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J38" s="2">
         <v>4</v>
@@ -2913,7 +2909,7 @@
         <v>-2</v>
       </c>
       <c r="T38" s="2">
-        <f>O38+P38+Q38+R38+S38</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U38" s="2">
@@ -2925,27 +2921,27 @@
     </row>
     <row r="39" spans="1:22" ht="56.25">
       <c r="A39" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J39" s="2">
         <v>4</v>
@@ -2972,32 +2968,32 @@
         <v>-2</v>
       </c>
       <c r="T39" s="2">
-        <f>O39+P39+Q39+R39+S39</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U39" s="2"/>
       <c r="V39" s="2"/>
     </row>
-    <row r="40" spans="1:22" ht="33.75">
+    <row r="40" spans="1:22" ht="33.75" hidden="1">
       <c r="A40" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2">
@@ -3025,7 +3021,7 @@
         <v>-2</v>
       </c>
       <c r="T40" s="2">
-        <f>O40+P40+Q40+R40+S40</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="U40" s="2"/>
@@ -3033,27 +3029,27 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:22" ht="157.5">
+    <row r="41" spans="1:22" ht="157.5" hidden="1">
       <c r="A41" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H41" s="2"/>
       <c r="I41" s="2"/>
@@ -3082,16 +3078,24 @@
         <v>-1</v>
       </c>
       <c r="T41" s="2">
-        <f>O41+P41+Q41+R41+S41</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="U41" s="2"/>
+      <c r="U41" s="2">
+        <v>2</v>
+      </c>
       <c r="V41" s="2">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V41"/>
+  <autoFilter ref="A1:V41">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Cavalry / Leaper"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Price promotion as an option
A promotable piece carries a premium: the gain promotion would bring it
over the distance it has to cross, times a factor to be tuned in
playtesting. Every Infantry piece holds the far-edge option too, priced
as a promotion into a Rook over six rows; it pays the higher of the
two. The sheet computes the premium from the promoted piece's own value,
with the factor, the far-edge stand-in and its distance as named
settings, and is sorted by value again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -10,14 +10,17 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$V$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$41</definedName>
+    <definedName name="PremiumFactor">Sheet1!$AA$2</definedName>
+    <definedName name="FarEdgeTarget">Sheet1!$AA$3</definedName>
+    <definedName name="FarEdgeDistance">Sheet1!$AA$4</definedName>
   </definedNames>
-  <calcPr calcId="114210"/>
+  <calcPr fullCalcOnLoad="1" calcId="114210"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="139">
   <si>
     <t>Piece Class</t>
   </si>
@@ -410,6 +413,30 @@
   </si>
   <si>
     <t>Reach (cells it could reach from d4 on an empty 8×8 board)</t>
+  </si>
+  <si>
+    <t>Promotion premium (gain ÷ distance × PremiumFactor; Infantry at least the far-edge option)</t>
+  </si>
+  <si>
+    <t>Own promotion (best)</t>
+  </si>
+  <si>
+    <t>Distance to own promotion (rows on 8×8)</t>
+  </si>
+  <si>
+    <t>Setting</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>PremiumFactor</t>
+  </si>
+  <si>
+    <t>FarEdgeTarget</t>
+  </si>
+  <si>
+    <t>FarEdgeDistance</t>
   </si>
 </sst>
 </file>
@@ -802,7 +829,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:V41"/>
+  <dimension ref="A1:AA41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="6"/>
@@ -810,7 +837,7 @@
     <col min="12" max="12" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="4" customFormat="1" ht="67.5">
+    <row r="1" spans="1:26" s="4" customFormat="1" ht="67.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -860,7 +887,7 @@
         <v>130</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
       <c r="R1" s="3" t="s">
         <v>16</v>
@@ -877,8 +904,20 @@
       <c r="V1" s="3" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" ht="33.75" hidden="1">
+      <c r="W1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="X1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" ht="33.75" hidden="1">
       <c r="A2" s="5" t="s">
         <v>21</v>
       </c>
@@ -916,6 +955,7 @@
         <v>18</v>
       </c>
       <c r="Q2" s="2">
+        <f>ROUND(MAX(0,IF(W2="",0,(VLOOKUP(W2,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/X2),IF(AND(A2="Infantry",ISERROR(SEARCH("Confined",E2))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R2" s="2">
@@ -925,13 +965,19 @@
         <v>0</v>
       </c>
       <c r="T2" s="2">
-        <f t="shared" ref="T2:T41" si="0">O2+P2+Q2+R2+S2</f>
+        <f>O2+P2+Q2+R2+S2</f>
         <v>78</v>
       </c>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
-    </row>
-    <row r="3" spans="1:22" ht="33.75" hidden="1">
+      <c r="Z2" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="AA2" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" ht="33.75" hidden="1">
       <c r="A3" s="5" t="s">
         <v>21</v>
       </c>
@@ -971,6 +1017,7 @@
         <v>16</v>
       </c>
       <c r="Q3" s="2">
+        <f>ROUND(MAX(0,IF(W3="",0,(VLOOKUP(W3,$B$2:$T$41,19,FALSE)-(O3+P3+R3+S3))/X3),IF(AND(A3="Infantry",ISERROR(SEARCH("Confined",E3))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O3+P3+R3+S3))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R3" s="2">
@@ -980,13 +1027,19 @@
         <v>0</v>
       </c>
       <c r="T3" s="2">
-        <f t="shared" si="0"/>
+        <f>O3+P3+Q3+R3+S3</f>
         <v>76</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:22" ht="22.5" hidden="1">
+      <c r="Z3" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="AA3" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" ht="22.5" hidden="1">
       <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
@@ -1026,6 +1079,7 @@
         <v>8</v>
       </c>
       <c r="Q4" s="2">
+        <f>ROUND(MAX(0,IF(W4="",0,(VLOOKUP(W4,$B$2:$T$41,19,FALSE)-(O4+P4+R4+S4))/X4),IF(AND(A4="Infantry",ISERROR(SEARCH("Confined",E4))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O4+P4+R4+S4))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R4" s="2">
@@ -1035,13 +1089,19 @@
         <v>0</v>
       </c>
       <c r="T4" s="2">
-        <f t="shared" si="0"/>
+        <f>O4+P4+Q4+R4+S4</f>
         <v>70</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
-    </row>
-    <row r="5" spans="1:22" ht="33.75" hidden="1">
+      <c r="Z4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="AA4" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" ht="33.75" hidden="1">
       <c r="A5" s="5" t="s">
         <v>21</v>
       </c>
@@ -1081,6 +1141,7 @@
         <v>4</v>
       </c>
       <c r="Q5" s="2">
+        <f>ROUND(MAX(0,IF(W5="",0,(VLOOKUP(W5,$B$2:$T$41,19,FALSE)-(O5+P5+R5+S5))/X5),IF(AND(A5="Infantry",ISERROR(SEARCH("Confined",E5))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O5+P5+R5+S5))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R5" s="2">
@@ -1090,7 +1151,7 @@
         <v>-2</v>
       </c>
       <c r="T5" s="2">
-        <f t="shared" si="0"/>
+        <f>O5+P5+Q5+R5+S5</f>
         <v>69</v>
       </c>
       <c r="U5" s="2"/>
@@ -1098,18 +1159,20 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:22" ht="78.75" hidden="1">
+    <row r="6" spans="1:26" ht="33.75" hidden="1">
       <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>127</v>
+        <v>71</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="E6" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="F6" s="2" t="s">
         <v>109</v>
       </c>
@@ -1121,54 +1184,53 @@
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K6" s="2">
         <v>1</v>
       </c>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N6" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="L6" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
       <c r="O6" s="2">
         <v>60</v>
       </c>
       <c r="P6" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q6" s="2">
+        <f>ROUND(MAX(0,IF(W6="",0,(VLOOKUP(W6,$B$2:$T$41,19,FALSE)-(O6+P6+R6+S6))/X6),IF(AND(A6="Infantry",ISERROR(SEARCH("Confined",E6))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O6+P6+R6+S6))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R6" s="2">
+        <v>2</v>
+      </c>
+      <c r="S6" s="2">
+        <v>-2</v>
+      </c>
+      <c r="T6" s="2">
+        <f>O6+P6+Q6+R6+S6</f>
+        <v>68</v>
+      </c>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2">
         <v>5</v>
       </c>
-      <c r="Q6" s="2">
-        <v>3</v>
-      </c>
-      <c r="R6" s="2">
-        <v>0</v>
-      </c>
-      <c r="S6" s="2">
-        <v>0</v>
-      </c>
-      <c r="T6" s="2">
-        <f t="shared" si="0"/>
-        <v>68</v>
-      </c>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-    </row>
-    <row r="7" spans="1:22" ht="33.75" hidden="1">
+    </row>
+    <row r="7" spans="1:26" ht="33.75" hidden="1">
       <c r="A7" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D7" s="2"/>
-      <c r="E7" s="2" t="s">
-        <v>103</v>
-      </c>
+      <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
         <v>109</v>
       </c>
@@ -1180,49 +1242,46 @@
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" s="2">
         <v>1</v>
       </c>
-      <c r="L7" s="2" t="s">
-        <v>116</v>
-      </c>
+      <c r="L7" s="2"/>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2">
         <v>60</v>
       </c>
       <c r="P7" s="2">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="Q7" s="2">
+        <f>ROUND(MAX(0,IF(W7="",0,(VLOOKUP(W7,$B$2:$T$41,19,FALSE)-(O7+P7+R7+S7))/X7),IF(AND(A7="Infantry",ISERROR(SEARCH("Confined",E7))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O7+P7+R7+S7))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R7" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="T7" s="2">
-        <f t="shared" si="0"/>
-        <v>68</v>
+        <f>O7+P7+Q7+R7+S7</f>
+        <v>66</v>
       </c>
       <c r="U7" s="2"/>
-      <c r="V7" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" ht="33.75" hidden="1">
+      <c r="V7" s="2"/>
+    </row>
+    <row r="8" spans="1:26" ht="78.75" hidden="1">
       <c r="A8" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>72</v>
+        <v>127</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -1237,21 +1296,26 @@
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K8" s="2">
         <v>1</v>
       </c>
       <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
+      <c r="M8" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="O8" s="2">
         <v>60</v>
       </c>
       <c r="P8" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="2">
+        <f>ROUND(MAX(0,IF(W8="",0,(VLOOKUP(W8,$B$2:$T$41,19,FALSE)-(O8+P8+R8+S8))/X8),IF(AND(A8="Infantry",ISERROR(SEARCH("Confined",E8))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O8+P8+R8+S8))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R8" s="2">
@@ -1261,13 +1325,19 @@
         <v>0</v>
       </c>
       <c r="T8" s="2">
-        <f t="shared" si="0"/>
-        <v>66</v>
+        <f>O8+P8+Q8+R8+S8</f>
+        <v>65</v>
       </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
-    </row>
-    <row r="9" spans="1:22" ht="33.75" hidden="1">
+      <c r="W8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X8" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" ht="33.75" hidden="1">
       <c r="A9" s="5" t="s">
         <v>23</v>
       </c>
@@ -1307,6 +1377,7 @@
         <v>35</v>
       </c>
       <c r="Q9" s="2">
+        <f>ROUND(MAX(0,IF(W9="",0,(VLOOKUP(W9,$B$2:$T$41,19,FALSE)-(O9+P9+R9+S9))/X9),IF(AND(A9="Infantry",ISERROR(SEARCH("Confined",E9))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O9+P9+R9+S9))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R9" s="2">
@@ -1316,13 +1387,13 @@
         <v>0</v>
       </c>
       <c r="T9" s="2">
-        <f t="shared" si="0"/>
+        <f>O9+P9+Q9+R9+S9</f>
         <v>37</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
     </row>
-    <row r="10" spans="1:22" ht="22.5" hidden="1">
+    <row r="10" spans="1:26" ht="22.5" hidden="1">
       <c r="A10" s="5" t="s">
         <v>23</v>
       </c>
@@ -1360,6 +1431,7 @@
         <v>27</v>
       </c>
       <c r="Q10" s="2">
+        <f>ROUND(MAX(0,IF(W10="",0,(VLOOKUP(W10,$B$2:$T$41,19,FALSE)-(O10+P10+R10+S10))/X10),IF(AND(A10="Infantry",ISERROR(SEARCH("Confined",E10))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O10+P10+R10+S10))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R10" s="2">
@@ -1369,13 +1441,13 @@
         <v>0</v>
       </c>
       <c r="T10" s="2">
-        <f t="shared" si="0"/>
+        <f>O10+P10+Q10+R10+S10</f>
         <v>27</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:22" ht="33.75" hidden="1">
+    <row r="11" spans="1:26" ht="33.75" hidden="1">
       <c r="A11" s="5" t="s">
         <v>23</v>
       </c>
@@ -1413,6 +1485,7 @@
         <v>22</v>
       </c>
       <c r="Q11" s="2">
+        <f>ROUND(MAX(0,IF(W11="",0,(VLOOKUP(W11,$B$2:$T$41,19,FALSE)-(O11+P11+R11+S11))/X11),IF(AND(A11="Infantry",ISERROR(SEARCH("Confined",E11))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O11+P11+R11+S11))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R11" s="2">
@@ -1422,13 +1495,13 @@
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <f t="shared" si="0"/>
+        <f>O11+P11+Q11+R11+S11</f>
         <v>22</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:22" ht="22.5" hidden="1">
+    <row r="12" spans="1:26" ht="22.5" hidden="1">
       <c r="A12" s="5" t="s">
         <v>23</v>
       </c>
@@ -1466,6 +1539,7 @@
         <v>21</v>
       </c>
       <c r="Q12" s="2">
+        <f>ROUND(MAX(0,IF(W12="",0,(VLOOKUP(W12,$B$2:$T$41,19,FALSE)-(O12+P12+R12+S12))/X12),IF(AND(A12="Infantry",ISERROR(SEARCH("Confined",E12))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O12+P12+R12+S12))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R12" s="2">
@@ -1475,13 +1549,13 @@
         <v>0</v>
       </c>
       <c r="T12" s="2">
-        <f t="shared" si="0"/>
+        <f>O12+P12+Q12+R12+S12</f>
         <v>21</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:22" ht="33.75" hidden="1">
+    <row r="13" spans="1:26" ht="33.75" hidden="1">
       <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
@@ -1519,6 +1593,7 @@
         <v>21</v>
       </c>
       <c r="Q13" s="2">
+        <f>ROUND(MAX(0,IF(W13="",0,(VLOOKUP(W13,$B$2:$T$41,19,FALSE)-(O13+P13+R13+S13))/X13),IF(AND(A13="Infantry",ISERROR(SEARCH("Confined",E13))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O13+P13+R13+S13))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R13" s="2">
@@ -1528,13 +1603,13 @@
         <v>0</v>
       </c>
       <c r="T13" s="2">
-        <f t="shared" si="0"/>
+        <f>O13+P13+Q13+R13+S13</f>
         <v>21</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:22" ht="33.75" hidden="1">
+    <row r="14" spans="1:26" ht="33.75" hidden="1">
       <c r="A14" s="5" t="s">
         <v>23</v>
       </c>
@@ -1572,6 +1647,7 @@
         <v>17</v>
       </c>
       <c r="Q14" s="2">
+        <f>ROUND(MAX(0,IF(W14="",0,(VLOOKUP(W14,$B$2:$T$41,19,FALSE)-(O14+P14+R14+S14))/X14),IF(AND(A14="Infantry",ISERROR(SEARCH("Confined",E14))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O14+P14+R14+S14))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R14" s="2">
@@ -1581,23 +1657,25 @@
         <v>0</v>
       </c>
       <c r="T14" s="2">
-        <f t="shared" si="0"/>
+        <f>O14+P14+Q14+R14+S14</f>
         <v>17</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:22" ht="22.5" hidden="1">
+    <row r="15" spans="1:26" ht="78.75" hidden="1">
       <c r="A15" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D15" s="2"/>
+        <v>88</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>101</v>
+      </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
         <v>109</v>
@@ -1608,112 +1686,134 @@
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="O15" s="2">
+        <v>0</v>
+      </c>
+      <c r="P15" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="2">
+        <f>ROUND(MAX(0,IF(W15="",0,(VLOOKUP(W15,$B$2:$T$41,19,FALSE)-(O15+P15+R15+S15))/X15),IF(AND(A15="Infantry",ISERROR(SEARCH("Confined",E15))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O15+P15+R15+S15))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>17</v>
+      </c>
+      <c r="R15" s="2">
+        <v>0</v>
+      </c>
+      <c r="S15" s="2">
+        <v>-1</v>
+      </c>
+      <c r="T15" s="2">
+        <f>O15+P15+Q15+R15+S15</f>
+        <v>17</v>
+      </c>
+      <c r="U15" s="2">
+        <v>2</v>
+      </c>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X15" s="2">
         <v>4</v>
       </c>
-      <c r="K15" s="2">
-        <v>7</v>
-      </c>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2">
-        <v>0</v>
-      </c>
-      <c r="P15" s="2">
-        <v>14</v>
-      </c>
-      <c r="Q15" s="2">
-        <v>0</v>
-      </c>
-      <c r="R15" s="2">
-        <v>0</v>
-      </c>
-      <c r="S15" s="2">
-        <v>0</v>
-      </c>
-      <c r="T15" s="2">
-        <f t="shared" si="0"/>
-        <v>14</v>
-      </c>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-    </row>
-    <row r="16" spans="1:22" ht="157.5">
+    </row>
+    <row r="16" spans="1:26" ht="78.75" hidden="1">
       <c r="A16" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G16" s="2"/>
+      <c r="G16" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="H16" s="2"/>
-      <c r="I16" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="I16" s="2"/>
       <c r="J16" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K16" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
+      <c r="M16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>122</v>
+      </c>
       <c r="O16" s="2">
         <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Q16" s="2">
-        <v>0</v>
+        <f>ROUND(MAX(0,IF(W16="",0,(VLOOKUP(W16,$B$2:$T$41,19,FALSE)-(O16+P16+R16+S16))/X16),IF(AND(A16="Infantry",ISERROR(SEARCH("Confined",E16))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O16+P16+R16+S16))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>13</v>
       </c>
       <c r="R16" s="2">
         <v>0</v>
       </c>
       <c r="S16" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T16" s="2">
-        <f t="shared" si="0"/>
-        <v>12</v>
+        <f>O16+P16+Q16+R16+S16</f>
+        <v>16</v>
       </c>
       <c r="U16" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V16" s="2"/>
-    </row>
-    <row r="17" spans="1:22" ht="45" hidden="1">
+      <c r="W16" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X16" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" ht="22.5" hidden="1">
       <c r="A17" s="5" t="s">
         <v>23</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="G17" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H17" s="2"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2">
         <v>4</v>
@@ -1728,49 +1828,52 @@
         <v>0</v>
       </c>
       <c r="P17" s="2">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q17" s="2">
+        <f>ROUND(MAX(0,IF(W17="",0,(VLOOKUP(W17,$B$2:$T$41,19,FALSE)-(O17+P17+R17+S17))/X17),IF(AND(A17="Infantry",ISERROR(SEARCH("Confined",E17))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O17+P17+R17+S17))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R17" s="2">
         <v>0</v>
       </c>
       <c r="S17" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T17" s="2">
-        <f t="shared" si="0"/>
-        <v>12</v>
+        <f>O17+P17+Q17+R17+S17</f>
+        <v>14</v>
       </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:22" ht="112.5" hidden="1">
+    <row r="18" spans="1:26" ht="157.5">
       <c r="A18" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="2"/>
+        <v>74</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>93</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="G18" s="2"/>
       <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
+      <c r="I18" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J18" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K18" s="2">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L18" s="2"/>
       <c r="M18" s="2"/>
@@ -1779,48 +1882,49 @@
         <v>0</v>
       </c>
       <c r="P18" s="2">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="Q18" s="2">
+        <f>ROUND(MAX(0,IF(W18="",0,(VLOOKUP(W18,$B$2:$T$41,19,FALSE)-(O18+P18+R18+S18))/X18),IF(AND(A18="Infantry",ISERROR(SEARCH("Confined",E18))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O18+P18+R18+S18))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R18" s="2">
         <v>0</v>
       </c>
       <c r="S18" s="2">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="T18" s="2">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="U18" s="2"/>
+        <f>O18+P18+Q18+R18+S18</f>
+        <v>12</v>
+      </c>
+      <c r="U18" s="2">
+        <v>3</v>
+      </c>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:22" ht="112.5" hidden="1">
+    <row r="19" spans="1:26" ht="45" hidden="1">
       <c r="A19" s="5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E19" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="F19" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G19" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="I19" s="2"/>
       <c r="J19" s="2">
         <v>4</v>
       </c>
@@ -1834,51 +1938,50 @@
         <v>0</v>
       </c>
       <c r="P19" s="2">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q19" s="2">
+        <f>ROUND(MAX(0,IF(W19="",0,(VLOOKUP(W19,$B$2:$T$41,19,FALSE)-(O19+P19+R19+S19))/X19),IF(AND(A19="Infantry",ISERROR(SEARCH("Confined",E19))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O19+P19+R19+S19))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R19" s="2">
         <v>0</v>
       </c>
       <c r="S19" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="T19" s="2">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="U19" s="2">
-        <v>3</v>
-      </c>
+        <f>O19+P19+Q19+R19+S19</f>
+        <v>12</v>
+      </c>
+      <c r="U19" s="2"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:22" ht="22.5">
+    <row r="20" spans="1:26" ht="112.5" hidden="1">
       <c r="A20" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G20" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="H20" s="2"/>
-      <c r="I20" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="I20" s="2"/>
       <c r="J20" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K20" s="2">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
@@ -1887,49 +1990,54 @@
         <v>0</v>
       </c>
       <c r="P20" s="2">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="Q20" s="2">
+        <f>ROUND(MAX(0,IF(W20="",0,(VLOOKUP(W20,$B$2:$T$41,19,FALSE)-(O20+P20+R20+S20))/X20),IF(AND(A20="Infantry",ISERROR(SEARCH("Confined",E20))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O20+P20+R20+S20))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R20" s="2">
         <v>0</v>
       </c>
       <c r="S20" s="2">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="T20" s="2">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <f>O20+P20+Q20+R20+S20</f>
+        <v>10</v>
       </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:22" ht="22.5">
+    <row r="21" spans="1:26" ht="112.5" hidden="1">
       <c r="A21" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>129</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G21" s="2"/>
+      <c r="G21" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
         <v>112</v>
       </c>
       <c r="J21" s="2">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K21" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -1938,108 +2046,96 @@
         <v>0</v>
       </c>
       <c r="P21" s="2">
+        <v>10</v>
+      </c>
+      <c r="Q21" s="2">
+        <f>ROUND(MAX(0,IF(W21="",0,(VLOOKUP(W21,$B$2:$T$41,19,FALSE)-(O21+P21+R21+S21))/X21),IF(AND(A21="Infantry",ISERROR(SEARCH("Confined",E21))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O21+P21+R21+S21))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R21" s="2">
+        <v>0</v>
+      </c>
+      <c r="S21" s="2">
+        <v>-2</v>
+      </c>
+      <c r="T21" s="2">
+        <f>O21+P21+Q21+R21+S21</f>
         <v>8</v>
       </c>
-      <c r="Q21" s="2">
-        <v>0</v>
-      </c>
-      <c r="R21" s="2">
-        <v>0</v>
-      </c>
-      <c r="S21" s="2">
-        <v>0</v>
-      </c>
-      <c r="T21" s="2">
-        <f t="shared" si="0"/>
-        <v>8</v>
-      </c>
-      <c r="U21" s="2"/>
+      <c r="U21" s="2">
+        <v>3</v>
+      </c>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:22" ht="123.75" hidden="1">
+    <row r="22" spans="1:26" ht="22.5">
       <c r="A22" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>98</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G22" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="G22" s="2"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
+      <c r="I22" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J22" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K22" s="2">
-        <v>1</v>
-      </c>
-      <c r="L22" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="N22" s="2" t="s">
-        <v>123</v>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
+      <c r="N22" s="2"/>
       <c r="O22" s="2">
         <v>0</v>
       </c>
       <c r="P22" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="Q22" s="2">
-        <v>5</v>
+        <f>ROUND(MAX(0,IF(W22="",0,(VLOOKUP(W22,$B$2:$T$41,19,FALSE)-(O22+P22+R22+S22))/X22),IF(AND(A22="Infantry",ISERROR(SEARCH("Confined",E22))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O22+P22+R22+S22))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
       </c>
       <c r="R22" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S22" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T22" s="2">
-        <f t="shared" si="0"/>
+        <f>O22+P22+Q22+R22+S22</f>
         <v>8</v>
       </c>
-      <c r="U22" s="2">
-        <v>2</v>
-      </c>
+      <c r="U22" s="2"/>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:22" ht="112.5" hidden="1">
+    <row r="23" spans="1:26" ht="22.5">
       <c r="A23" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="G23" s="2"/>
+      <c r="H23" s="2"/>
       <c r="I23" s="2" t="s">
         <v>112</v>
       </c>
@@ -2047,7 +2143,7 @@
         <v>8</v>
       </c>
       <c r="K23" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -2059,95 +2155,113 @@
         <v>8</v>
       </c>
       <c r="Q23" s="2">
+        <f>ROUND(MAX(0,IF(W23="",0,(VLOOKUP(W23,$B$2:$T$41,19,FALSE)-(O23+P23+R23+S23))/X23),IF(AND(A23="Infantry",ISERROR(SEARCH("Confined",E23))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O23+P23+R23+S23))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R23" s="2">
         <v>0</v>
       </c>
       <c r="S23" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T23" s="2">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="U23" s="2">
+        <f>O23+P23+Q23+R23+S23</f>
+        <v>8</v>
+      </c>
+      <c r="U23" s="2"/>
+      <c r="V23" s="2"/>
+    </row>
+    <row r="24" spans="1:26" ht="123.75" hidden="1">
+      <c r="A24" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H24" s="2"/>
+      <c r="I24" s="2"/>
+      <c r="J24" s="2">
         <v>3</v>
       </c>
-      <c r="V23" s="2"/>
-    </row>
-    <row r="24" spans="1:22" ht="45">
-      <c r="A24" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J24" s="2">
-        <v>8</v>
-      </c>
       <c r="K24" s="2">
+        <v>1</v>
+      </c>
+      <c r="L24" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="O24" s="2">
+        <v>0</v>
+      </c>
+      <c r="P24" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q24" s="2">
+        <f>ROUND(MAX(0,IF(W24="",0,(VLOOKUP(W24,$B$2:$T$41,19,FALSE)-(O24+P24+R24+S24))/X24),IF(AND(A24="Infantry",ISERROR(SEARCH("Confined",E24))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O24+P24+R24+S24))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>4</v>
       </c>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2">
-        <v>0</v>
-      </c>
-      <c r="P24" s="2">
-        <v>8</v>
-      </c>
-      <c r="Q24" s="2">
-        <v>0</v>
-      </c>
       <c r="R24" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S24" s="2">
         <v>-1</v>
       </c>
       <c r="T24" s="2">
-        <f t="shared" si="0"/>
+        <f>O24+P24+Q24+R24+S24</f>
         <v>7</v>
       </c>
-      <c r="U24" s="2"/>
+      <c r="U24" s="2">
+        <v>2</v>
+      </c>
       <c r="V24" s="2"/>
-    </row>
-    <row r="25" spans="1:22" ht="90">
+      <c r="W24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X24" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:26" ht="112.5" hidden="1">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G25" s="2"/>
-      <c r="H25" s="2"/>
+      <c r="G25" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I25" s="2" t="s">
         <v>112</v>
       </c>
@@ -2155,7 +2269,7 @@
         <v>8</v>
       </c>
       <c r="K25" s="2">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -2167,6 +2281,7 @@
         <v>8</v>
       </c>
       <c r="Q25" s="2">
+        <f>ROUND(MAX(0,IF(W25="",0,(VLOOKUP(W25,$B$2:$T$41,19,FALSE)-(O25+P25+R25+S25))/X25),IF(AND(A25="Infantry",ISERROR(SEARCH("Confined",E25))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O25+P25+R25+S25))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R25" s="2">
@@ -2176,43 +2291,41 @@
         <v>-1</v>
       </c>
       <c r="T25" s="2">
-        <f t="shared" si="0"/>
+        <f>O25+P25+Q25+R25+S25</f>
         <v>7</v>
       </c>
       <c r="U25" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V25" s="2"/>
     </row>
-    <row r="26" spans="1:22" ht="101.25">
+    <row r="26" spans="1:26" ht="45">
       <c r="A26" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E26" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="F26" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="I26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+      <c r="I26" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J26" s="2">
         <v>8</v>
       </c>
       <c r="K26" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -2224,6 +2337,7 @@
         <v>8</v>
       </c>
       <c r="Q26" s="2">
+        <f>ROUND(MAX(0,IF(W26="",0,(VLOOKUP(W26,$B$2:$T$41,19,FALSE)-(O26+P26+R26+S26))/X26),IF(AND(A26="Infantry",ISERROR(SEARCH("Confined",E26))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O26+P26+R26+S26))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R26" s="2">
@@ -2233,47 +2347,41 @@
         <v>-1</v>
       </c>
       <c r="T26" s="2">
-        <f t="shared" si="0"/>
+        <f>O26+P26+Q26+R26+S26</f>
         <v>7</v>
       </c>
-      <c r="U26" s="2">
-        <v>2</v>
-      </c>
+      <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:22" ht="33.75" hidden="1">
+    <row r="27" spans="1:26" ht="90">
       <c r="A27" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D27" s="2"/>
-      <c r="E27" s="2" t="s">
-        <v>103</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G27" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="I27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+      <c r="I27" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J27" s="2">
         <v>8</v>
       </c>
       <c r="K27" s="2">
-        <v>1</v>
-      </c>
-      <c r="L27" s="2" t="s">
-        <v>118</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="L27" s="2"/>
       <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="2">
@@ -2283,35 +2391,36 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
+        <f>ROUND(MAX(0,IF(W27="",0,(VLOOKUP(W27,$B$2:$T$41,19,FALSE)-(O27+P27+R27+S27))/X27),IF(AND(A27="Infantry",ISERROR(SEARCH("Confined",E27))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O27+P27+R27+S27))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S27" s="2">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="T27" s="2">
-        <f t="shared" si="0"/>
+        <f>O27+P27+Q27+R27+S27</f>
         <v>7</v>
       </c>
-      <c r="U27" s="2"/>
-      <c r="V27" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:22" ht="78.75" hidden="1">
+      <c r="U27" s="2">
+        <v>2</v>
+      </c>
+      <c r="V27" s="2"/>
+    </row>
+    <row r="28" spans="1:26" ht="101.25">
       <c r="A28" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
@@ -2320,29 +2429,28 @@
       <c r="G28" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="H28" s="2"/>
+      <c r="H28" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K28" s="2">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="M28" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N28" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="M28" s="2"/>
+      <c r="N28" s="2"/>
       <c r="O28" s="2">
         <v>0</v>
       </c>
       <c r="P28" s="2">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="Q28" s="2">
-        <v>3</v>
+        <f>ROUND(MAX(0,IF(W28="",0,(VLOOKUP(W28,$B$2:$T$41,19,FALSE)-(O28+P28+R28+S28))/X28),IF(AND(A28="Infantry",ISERROR(SEARCH("Confined",E28))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O28+P28+R28+S28))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
       </c>
       <c r="R28" s="2">
         <v>0</v>
@@ -2351,26 +2459,28 @@
         <v>-1</v>
       </c>
       <c r="T28" s="2">
-        <f t="shared" si="0"/>
-        <v>6</v>
+        <f>O28+P28+Q28+R28+S28</f>
+        <v>7</v>
       </c>
       <c r="U28" s="2">
         <v>2</v>
       </c>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:22" ht="22.5" hidden="1">
+    <row r="29" spans="1:26" ht="33.75" hidden="1">
       <c r="A29" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>127</v>
+        <v>71</v>
       </c>
       <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="E29" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="F29" s="2" t="s">
         <v>109</v>
       </c>
@@ -2382,52 +2492,53 @@
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K29" s="2">
         <v>1</v>
       </c>
-      <c r="L29" s="2"/>
+      <c r="L29" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
       <c r="O29" s="2">
         <v>0</v>
       </c>
       <c r="P29" s="2">
+        <v>8</v>
+      </c>
+      <c r="Q29" s="2">
+        <f>ROUND(MAX(0,IF(W29="",0,(VLOOKUP(W29,$B$2:$T$41,19,FALSE)-(O29+P29+R29+S29))/X29),IF(AND(A29="Infantry",ISERROR(SEARCH("Confined",E29))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O29+P29+R29+S29))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
+      </c>
+      <c r="R29" s="2">
+        <v>1</v>
+      </c>
+      <c r="S29" s="2">
+        <v>-2</v>
+      </c>
+      <c r="T29" s="2">
+        <f>O29+P29+Q29+R29+S29</f>
+        <v>7</v>
+      </c>
+      <c r="U29" s="2"/>
+      <c r="V29" s="2">
         <v>5</v>
       </c>
-      <c r="Q29" s="2">
-        <v>0</v>
-      </c>
-      <c r="R29" s="2">
-        <v>0</v>
-      </c>
-      <c r="S29" s="2">
-        <v>0</v>
-      </c>
-      <c r="T29" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="U29" s="2"/>
-      <c r="V29" s="2"/>
-    </row>
-    <row r="30" spans="1:22" ht="90" hidden="1">
+    </row>
+    <row r="30" spans="1:26" ht="22.5" hidden="1">
       <c r="A30" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>107</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
         <v>109</v>
       </c>
@@ -2435,7 +2546,7 @@
         <v>112</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2">
@@ -2444,9 +2555,7 @@
       <c r="K30" s="2">
         <v>1</v>
       </c>
-      <c r="L30" s="2" t="s">
-        <v>119</v>
-      </c>
+      <c r="L30" s="2"/>
       <c r="M30" s="2"/>
       <c r="N30" s="2"/>
       <c r="O30" s="2">
@@ -2456,77 +2565,87 @@
         <v>5</v>
       </c>
       <c r="Q30" s="2">
-        <v>0</v>
+        <f>ROUND(MAX(0,IF(W30="",0,(VLOOKUP(W30,$B$2:$T$41,19,FALSE)-(O30+P30+R30+S30))/X30),IF(AND(A30="Infantry",ISERROR(SEARCH("Confined",E30))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O30+P30+R30+S30))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
       </c>
       <c r="R30" s="2">
+        <v>0</v>
+      </c>
+      <c r="S30" s="2">
+        <v>0</v>
+      </c>
+      <c r="T30" s="2">
+        <f>O30+P30+Q30+R30+S30</f>
+        <v>7</v>
+      </c>
+      <c r="U30" s="2"/>
+      <c r="V30" s="2"/>
+    </row>
+    <row r="31" spans="1:26" ht="90" hidden="1">
+      <c r="A31" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2">
+        <v>5</v>
+      </c>
+      <c r="K31" s="2">
         <v>1</v>
       </c>
-      <c r="S30" s="2">
-        <v>-1</v>
-      </c>
-      <c r="T30" s="2">
-        <f t="shared" si="0"/>
-        <v>5</v>
-      </c>
-      <c r="U30" s="2">
-        <v>2</v>
-      </c>
-      <c r="V30" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:22" ht="22.5">
-      <c r="A31" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J31" s="2">
-        <v>8</v>
-      </c>
-      <c r="K31" s="2">
-        <v>5</v>
-      </c>
-      <c r="L31" s="2"/>
+      <c r="L31" s="2" t="s">
+        <v>119</v>
+      </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
       <c r="O31" s="2">
         <v>0</v>
       </c>
       <c r="P31" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q31" s="2">
-        <v>0</v>
+        <f>ROUND(MAX(0,IF(W31="",0,(VLOOKUP(W31,$B$2:$T$41,19,FALSE)-(O31+P31+R31+S31))/X31),IF(AND(A31="Infantry",ISERROR(SEARCH("Confined",E31))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O31+P31+R31+S31))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
       </c>
       <c r="R31" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S31" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T31" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-    </row>
-    <row r="32" spans="1:22" hidden="1">
+        <f>O31+P31+Q31+R31+S31</f>
+        <v>7</v>
+      </c>
+      <c r="U31" s="2">
+        <v>2</v>
+      </c>
+      <c r="V31" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:26" hidden="1">
       <c r="A32" s="5" t="s">
         <v>22</v>
       </c>
@@ -2562,7 +2681,8 @@
         <v>4</v>
       </c>
       <c r="Q32" s="2">
-        <v>0</v>
+        <f>ROUND(MAX(0,IF(W32="",0,(VLOOKUP(W32,$B$2:$T$41,19,FALSE)-(O32+P32+R32+S32))/X32),IF(AND(A32="Infantry",ISERROR(SEARCH("Confined",E32))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O32+P32+R32+S32))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
       </c>
       <c r="R32" s="2">
         <v>0</v>
@@ -2571,55 +2691,52 @@
         <v>0</v>
       </c>
       <c r="T32" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <f>O32+P32+Q32+R32+S32</f>
+        <v>6</v>
       </c>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:22" ht="78.75" hidden="1">
+    <row r="33" spans="1:26" ht="45" hidden="1">
       <c r="A33" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="E33" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="F33" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G33" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K33" s="2">
         <v>1</v>
       </c>
       <c r="L33" s="2"/>
-      <c r="M33" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="N33" s="2" t="s">
-        <v>122</v>
-      </c>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
       <c r="O33" s="2">
         <v>0</v>
       </c>
       <c r="P33" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q33" s="2">
-        <v>4</v>
+        <f>ROUND(MAX(0,IF(W33="",0,(VLOOKUP(W33,$B$2:$T$41,19,FALSE)-(O33+P33+R33+S33))/X33),IF(AND(A33="Infantry",ISERROR(SEARCH("Confined",E33))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O33+P33+R33+S33))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
       </c>
       <c r="R33" s="2">
         <v>0</v>
@@ -2628,112 +2745,108 @@
         <v>-1</v>
       </c>
       <c r="T33" s="2">
-        <f t="shared" si="0"/>
-        <v>4</v>
-      </c>
-      <c r="U33" s="2">
-        <v>2</v>
-      </c>
+        <f>O33+P33+Q33+R33+S33</f>
+        <v>5</v>
+      </c>
+      <c r="U33" s="2"/>
       <c r="V33" s="2"/>
     </row>
-    <row r="34" spans="1:22" ht="78.75" hidden="1">
+    <row r="34" spans="1:26" ht="22.5">
       <c r="A34" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>101</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="G34" s="2"/>
       <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
+      <c r="I34" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J34" s="2">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="K34" s="2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L34" s="2"/>
-      <c r="M34" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>124</v>
-      </c>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
       <c r="O34" s="2">
         <v>0</v>
       </c>
       <c r="P34" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q34" s="2">
-        <v>1</v>
+        <f>ROUND(MAX(0,IF(W34="",0,(VLOOKUP(W34,$B$2:$T$41,19,FALSE)-(O34+P34+R34+S34))/X34),IF(AND(A34="Infantry",ISERROR(SEARCH("Confined",E34))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O34+P34+R34+S34))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>0</v>
       </c>
       <c r="R34" s="2">
         <v>0</v>
       </c>
       <c r="S34" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T34" s="2">
-        <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="U34" s="2">
-        <v>2</v>
-      </c>
+        <f>O34+P34+Q34+R34+S34</f>
+        <v>4</v>
+      </c>
+      <c r="U34" s="2"/>
       <c r="V34" s="2"/>
     </row>
-    <row r="35" spans="1:22" ht="45" hidden="1">
+    <row r="35" spans="1:26" ht="78.75" hidden="1">
       <c r="A35" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" s="2"/>
       <c r="F35" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K35" s="2">
         <v>1</v>
       </c>
       <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2"/>
+      <c r="M35" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O35" s="2">
         <v>0</v>
       </c>
       <c r="P35" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q35" s="2">
-        <v>0</v>
+        <f>ROUND(MAX(0,IF(W35="",0,(VLOOKUP(W35,$B$2:$T$41,19,FALSE)-(O35+P35+R35+S35))/X35),IF(AND(A35="Infantry",ISERROR(SEARCH("Confined",E35))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O35+P35+R35+S35))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
       </c>
       <c r="R35" s="2">
         <v>0</v>
@@ -2742,41 +2855,49 @@
         <v>-1</v>
       </c>
       <c r="T35" s="2">
-        <f t="shared" si="0"/>
+        <f>O35+P35+Q35+R35+S35</f>
+        <v>4</v>
+      </c>
+      <c r="U35" s="2">
+        <v>2</v>
+      </c>
+      <c r="V35" s="2"/>
+      <c r="W35" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="X35" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:26" ht="157.5" hidden="1">
+      <c r="A36" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2">
         <v>3</v>
       </c>
-      <c r="U35" s="2"/>
-      <c r="V35" s="2"/>
-    </row>
-    <row r="36" spans="1:22" ht="45">
-      <c r="A36" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="G36" s="2"/>
-      <c r="H36" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="J36" s="2">
-        <v>4</v>
-      </c>
       <c r="K36" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
@@ -2785,45 +2906,50 @@
         <v>0</v>
       </c>
       <c r="P36" s="2">
+        <v>3</v>
+      </c>
+      <c r="Q36" s="2">
+        <f>ROUND(MAX(0,IF(W36="",0,(VLOOKUP(W36,$B$2:$T$41,19,FALSE)-(O36+P36+R36+S36))/X36),IF(AND(A36="Infantry",ISERROR(SEARCH("Confined",E36))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O36+P36+R36+S36))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <v>2</v>
+      </c>
+      <c r="R36" s="2">
+        <v>0</v>
+      </c>
+      <c r="S36" s="2">
+        <v>-1</v>
+      </c>
+      <c r="T36" s="2">
+        <f>O36+P36+Q36+R36+S36</f>
         <v>4</v>
       </c>
-      <c r="Q36" s="2">
-        <v>0</v>
-      </c>
-      <c r="R36" s="2">
-        <v>0</v>
-      </c>
-      <c r="S36" s="2">
-        <v>-2</v>
-      </c>
-      <c r="T36" s="2">
-        <f t="shared" si="0"/>
+      <c r="U36" s="2">
         <v>2</v>
       </c>
-      <c r="U36" s="2"/>
-      <c r="V36" s="2"/>
-    </row>
-    <row r="37" spans="1:22" ht="56.25">
+      <c r="V36" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:26" ht="45">
       <c r="A37" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G37" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H37" s="2"/>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I37" s="2" t="s">
         <v>112</v>
       </c>
@@ -2831,7 +2957,7 @@
         <v>4</v>
       </c>
       <c r="K37" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L37" s="2"/>
       <c r="M37" s="2"/>
@@ -2843,6 +2969,7 @@
         <v>4</v>
       </c>
       <c r="Q37" s="2">
+        <f>ROUND(MAX(0,IF(W37="",0,(VLOOKUP(W37,$B$2:$T$41,19,FALSE)-(O37+P37+R37+S37))/X37),IF(AND(A37="Infantry",ISERROR(SEARCH("Confined",E37))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O37+P37+R37+S37))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R37" s="2">
@@ -2852,35 +2979,33 @@
         <v>-2</v>
       </c>
       <c r="T37" s="2">
-        <f t="shared" si="0"/>
+        <f>O37+P37+Q37+R37+S37</f>
         <v>2</v>
       </c>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
     </row>
-    <row r="38" spans="1:22" ht="101.25">
+    <row r="38" spans="1:26" ht="56.25">
       <c r="A38" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>99</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G38" s="2"/>
-      <c r="H38" s="2" t="s">
-        <v>112</v>
-      </c>
+      <c r="G38" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H38" s="2"/>
       <c r="I38" s="2" t="s">
         <v>112</v>
       </c>
@@ -2888,7 +3013,7 @@
         <v>4</v>
       </c>
       <c r="K38" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
@@ -2900,6 +3025,7 @@
         <v>4</v>
       </c>
       <c r="Q38" s="2">
+        <f>ROUND(MAX(0,IF(W38="",0,(VLOOKUP(W38,$B$2:$T$41,19,FALSE)-(O38+P38+R38+S38))/X38),IF(AND(A38="Infantry",ISERROR(SEARCH("Confined",E38))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O38+P38+R38+S38))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R38" s="2">
@@ -2909,37 +3035,35 @@
         <v>-2</v>
       </c>
       <c r="T38" s="2">
-        <f t="shared" si="0"/>
+        <f>O38+P38+Q38+R38+S38</f>
         <v>2</v>
       </c>
-      <c r="U38" s="2">
-        <v>2</v>
-      </c>
-      <c r="V38" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:22" ht="56.25">
+      <c r="U38" s="2"/>
+      <c r="V38" s="2"/>
+    </row>
+    <row r="39" spans="1:26" ht="101.25">
       <c r="A39" s="5" t="s">
         <v>24</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="D39" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="E39" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G39" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H39" s="2"/>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I39" s="2" t="s">
         <v>112</v>
       </c>
@@ -2947,7 +3071,7 @@
         <v>4</v>
       </c>
       <c r="K39" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
@@ -2959,6 +3083,7 @@
         <v>4</v>
       </c>
       <c r="Q39" s="2">
+        <f>ROUND(MAX(0,IF(W39="",0,(VLOOKUP(W39,$B$2:$T$41,19,FALSE)-(O39+P39+R39+S39))/X39),IF(AND(A39="Infantry",ISERROR(SEARCH("Confined",E39))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O39+P39+R39+S39))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R39" s="2">
@@ -2968,39 +3093,45 @@
         <v>-2</v>
       </c>
       <c r="T39" s="2">
-        <f t="shared" si="0"/>
+        <f>O39+P39+Q39+R39+S39</f>
         <v>2</v>
       </c>
-      <c r="U39" s="2"/>
-      <c r="V39" s="2"/>
-    </row>
-    <row r="40" spans="1:22" ht="33.75" hidden="1">
+      <c r="U39" s="2">
+        <v>2</v>
+      </c>
+      <c r="V39" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:26" ht="56.25">
       <c r="A40" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>70</v>
+        <v>91</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="I40" s="2"/>
+      <c r="G40" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="J40" s="2">
         <v>4</v>
       </c>
       <c r="K40" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
@@ -3012,6 +3143,7 @@
         <v>4</v>
       </c>
       <c r="Q40" s="2">
+        <f>ROUND(MAX(0,IF(W40="",0,(VLOOKUP(W40,$B$2:$T$41,19,FALSE)-(O40+P40+R40+S40))/X40),IF(AND(A40="Infantry",ISERROR(SEARCH("Confined",E40))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O40+P40+R40+S40))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R40" s="2">
@@ -3021,40 +3153,36 @@
         <v>-2</v>
       </c>
       <c r="T40" s="2">
-        <f t="shared" si="0"/>
+        <f>O40+P40+Q40+R40+S40</f>
         <v>2</v>
       </c>
       <c r="U40" s="2"/>
-      <c r="V40" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:22" ht="157.5" hidden="1">
+      <c r="V40" s="2"/>
+    </row>
+    <row r="41" spans="1:26" ht="33.75" hidden="1">
       <c r="A41" s="5" t="s">
         <v>22</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>102</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F41" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="H41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K41" s="2">
         <v>1</v>
@@ -3066,30 +3194,29 @@
         <v>0</v>
       </c>
       <c r="P41" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q41" s="2">
+        <f>ROUND(MAX(0,IF(W41="",0,(VLOOKUP(W41,$B$2:$T$41,19,FALSE)-(O41+P41+R41+S41))/X41),IF(AND(A41="Infantry",ISERROR(SEARCH("Confined",E41))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O41+P41+R41+S41))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R41" s="2">
         <v>0</v>
       </c>
       <c r="S41" s="2">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="T41" s="2">
-        <f t="shared" si="0"/>
+        <f>O41+P41+Q41+R41+S41</f>
         <v>2</v>
       </c>
-      <c r="U41" s="2">
-        <v>2</v>
-      </c>
+      <c r="U41" s="2"/>
       <c r="V41" s="2">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V41">
+  <autoFilter ref="A1:X41">
     <filterColumn colId="0">
       <filters>
         <filter val="Cavalry / Leaper"/>

</xml_diff>

<commit_message>
Settle the last design questions, and call it a leader face-off
The proposals for the largest board, random ranges, rivers, start rows,
confinement, the flying-general capture and castling are agreed. A step
along a palace line goes to the next cell the line passes through, not
only through centres, which may be a setting. The Janggi General's power
becomes the leader face-off, since neither leader need be in a palace,
and it is offered, not automatic. Only a second palace, and what
playtesting is to settle, remain open.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -11,16 +11,16 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$41</definedName>
+    <definedName name="FarEdgeDistance">Sheet1!$AA$4</definedName>
+    <definedName name="FarEdgeTarget">Sheet1!$AA$3</definedName>
     <definedName name="PremiumFactor">Sheet1!$AA$2</definedName>
-    <definedName name="FarEdgeTarget">Sheet1!$AA$3</definedName>
-    <definedName name="FarEdgeDistance">Sheet1!$AA$4</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1" calcId="114210"/>
+  <calcPr calcId="114210"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="138">
   <si>
     <t>Piece Class</t>
   </si>
@@ -67,9 +67,6 @@
     <t>Leader bonus</t>
   </si>
   <si>
-    <t>Promotion bonus</t>
-  </si>
-  <si>
     <t>Special-power bonus</t>
   </si>
   <si>
@@ -370,7 +367,7 @@
     <t>Castling</t>
   </si>
   <si>
-    <t>Palace Face-Off; Can move diagonally along marked palace lines</t>
+    <t>Leader Face-Off; Can move diagonally along marked palace lines</t>
   </si>
   <si>
     <t>First move may advance two squares; en passant</t>
@@ -828,7 +825,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -837,7 +833,7 @@
     <col min="12" max="12" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" s="4" customFormat="1" ht="67.5">
+    <row r="1" spans="1:27" s="4" customFormat="1" ht="112.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -884,59 +880,59 @@
         <v>14</v>
       </c>
       <c r="P1" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="W1" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="R1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="33.75">
+      <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="W1" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" ht="33.75" hidden="1">
-      <c r="A2" s="5" t="s">
-        <v>21</v>
-      </c>
       <c r="B2" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2">
@@ -955,7 +951,7 @@
         <v>18</v>
       </c>
       <c r="Q2" s="2">
-        <f>ROUND(MAX(0,IF(W2="",0,(VLOOKUP(W2,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/X2),IF(AND(A2="Infantry",ISERROR(SEARCH("Confined",E2))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ref="Q2:Q41" ca="1" si="0">ROUND(MAX(0,IF(W2="",0,(VLOOKUP(W2,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/X2),IF(AND(A2="Infantry",ISERROR(SEARCH("Confined",E2))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O2+P2+R2+S2))/FarEdgeDistance,0))*PremiumFactor,0)</f>
         <v>0</v>
       </c>
       <c r="R2" s="2">
@@ -965,41 +961,41 @@
         <v>0</v>
       </c>
       <c r="T2" s="2">
-        <f>O2+P2+Q2+R2+S2</f>
+        <f t="shared" ref="T2:T41" si="1">O2+P2+Q2+R2+S2</f>
         <v>78</v>
       </c>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
       <c r="Z2" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AA2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="33.75" hidden="1">
+    <row r="3" spans="1:27" ht="33.75">
       <c r="A3" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J3" s="2">
         <v>8</v>
@@ -1017,7 +1013,7 @@
         <v>16</v>
       </c>
       <c r="Q3" s="2">
-        <f>ROUND(MAX(0,IF(W3="",0,(VLOOKUP(W3,$B$2:$T$41,19,FALSE)-(O3+P3+R3+S3))/X3),IF(AND(A3="Infantry",ISERROR(SEARCH("Confined",E3))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O3+P3+R3+S3))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R3" s="2">
@@ -1027,38 +1023,38 @@
         <v>0</v>
       </c>
       <c r="T3" s="2">
-        <f>O3+P3+Q3+R3+S3</f>
+        <f t="shared" si="1"/>
         <v>76</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="Z3" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" ht="22.5" hidden="1">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="22.5">
       <c r="A4" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
@@ -1068,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -1079,7 +1075,7 @@
         <v>8</v>
       </c>
       <c r="Q4" s="2">
-        <f>ROUND(MAX(0,IF(W4="",0,(VLOOKUP(W4,$B$2:$T$41,19,FALSE)-(O4+P4+R4+S4))/X4),IF(AND(A4="Infantry",ISERROR(SEARCH("Confined",E4))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O4+P4+R4+S4))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R4" s="2">
@@ -1089,37 +1085,37 @@
         <v>0</v>
       </c>
       <c r="T4" s="2">
-        <f>O4+P4+Q4+R4+S4</f>
+        <f t="shared" si="1"/>
         <v>70</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="Z4" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="AA4" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="33.75" hidden="1">
+    <row r="5" spans="1:27" ht="33.75">
       <c r="A5" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1130,7 +1126,7 @@
         <v>7</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1141,7 +1137,7 @@
         <v>4</v>
       </c>
       <c r="Q5" s="2">
-        <f>ROUND(MAX(0,IF(W5="",0,(VLOOKUP(W5,$B$2:$T$41,19,FALSE)-(O5+P5+R5+S5))/X5),IF(AND(A5="Infantry",ISERROR(SEARCH("Confined",E5))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O5+P5+R5+S5))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R5" s="2">
@@ -1151,7 +1147,7 @@
         <v>-2</v>
       </c>
       <c r="T5" s="2">
-        <f>O5+P5+Q5+R5+S5</f>
+        <f t="shared" si="1"/>
         <v>69</v>
       </c>
       <c r="U5" s="2"/>
@@ -1159,28 +1155,28 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="33.75" hidden="1">
+    <row r="6" spans="1:27" ht="33.75">
       <c r="A6" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
@@ -1190,7 +1186,7 @@
         <v>1</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -1201,7 +1197,7 @@
         <v>8</v>
       </c>
       <c r="Q6" s="2">
-        <f>ROUND(MAX(0,IF(W6="",0,(VLOOKUP(W6,$B$2:$T$41,19,FALSE)-(O6+P6+R6+S6))/X6),IF(AND(A6="Infantry",ISERROR(SEARCH("Confined",E6))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O6+P6+R6+S6))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R6" s="2">
@@ -1211,7 +1207,7 @@
         <v>-2</v>
       </c>
       <c r="T6" s="2">
-        <f>O6+P6+Q6+R6+S6</f>
+        <f t="shared" si="1"/>
         <v>68</v>
       </c>
       <c r="U6" s="2"/>
@@ -1219,26 +1215,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="33.75" hidden="1">
+    <row r="7" spans="1:27" ht="33.75">
       <c r="A7" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
@@ -1257,7 +1253,7 @@
         <v>6</v>
       </c>
       <c r="Q7" s="2">
-        <f>ROUND(MAX(0,IF(W7="",0,(VLOOKUP(W7,$B$2:$T$41,19,FALSE)-(O7+P7+R7+S7))/X7),IF(AND(A7="Infantry",ISERROR(SEARCH("Confined",E7))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O7+P7+R7+S7))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R7" s="2">
@@ -1267,32 +1263,32 @@
         <v>0</v>
       </c>
       <c r="T7" s="2">
-        <f>O7+P7+Q7+R7+S7</f>
+        <f t="shared" si="1"/>
         <v>66</v>
       </c>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
     </row>
-    <row r="8" spans="1:26" ht="78.75" hidden="1">
+    <row r="8" spans="1:27" ht="78.75">
       <c r="A8" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
@@ -1303,10 +1299,10 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O8" s="2">
         <v>60</v>
@@ -1315,7 +1311,7 @@
         <v>5</v>
       </c>
       <c r="Q8" s="2">
-        <f>ROUND(MAX(0,IF(W8="",0,(VLOOKUP(W8,$B$2:$T$41,19,FALSE)-(O8+P8+R8+S8))/X8),IF(AND(A8="Infantry",ISERROR(SEARCH("Confined",E8))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O8+P8+R8+S8))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R8" s="2">
@@ -1325,41 +1321,41 @@
         <v>0</v>
       </c>
       <c r="T8" s="2">
-        <f>O8+P8+Q8+R8+S8</f>
+        <f t="shared" si="1"/>
         <v>65</v>
       </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="X8" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="33.75" hidden="1">
+    <row r="9" spans="1:27" ht="33.75">
       <c r="A9" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J9" s="2">
         <v>8</v>
@@ -1377,7 +1373,7 @@
         <v>35</v>
       </c>
       <c r="Q9" s="2">
-        <f>ROUND(MAX(0,IF(W9="",0,(VLOOKUP(W9,$B$2:$T$41,19,FALSE)-(O9+P9+R9+S9))/X9),IF(AND(A9="Infantry",ISERROR(SEARCH("Confined",E9))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O9+P9+R9+S9))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R9" s="2">
@@ -1387,32 +1383,32 @@
         <v>0</v>
       </c>
       <c r="T9" s="2">
-        <f>O9+P9+Q9+R9+S9</f>
+        <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
     </row>
-    <row r="10" spans="1:26" ht="22.5" hidden="1">
+    <row r="10" spans="1:27" ht="22.5">
       <c r="A10" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2">
@@ -1431,7 +1427,7 @@
         <v>27</v>
       </c>
       <c r="Q10" s="2">
-        <f>ROUND(MAX(0,IF(W10="",0,(VLOOKUP(W10,$B$2:$T$41,19,FALSE)-(O10+P10+R10+S10))/X10),IF(AND(A10="Infantry",ISERROR(SEARCH("Confined",E10))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O10+P10+R10+S10))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R10" s="2">
@@ -1441,33 +1437,33 @@
         <v>0</v>
       </c>
       <c r="T10" s="2">
-        <f>O10+P10+Q10+R10+S10</f>
+        <f t="shared" si="1"/>
         <v>27</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:26" ht="33.75" hidden="1">
+    <row r="11" spans="1:27" ht="33.75">
       <c r="A11" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J11" s="2">
         <v>8</v>
@@ -1485,7 +1481,7 @@
         <v>22</v>
       </c>
       <c r="Q11" s="2">
-        <f>ROUND(MAX(0,IF(W11="",0,(VLOOKUP(W11,$B$2:$T$41,19,FALSE)-(O11+P11+R11+S11))/X11),IF(AND(A11="Infantry",ISERROR(SEARCH("Confined",E11))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O11+P11+R11+S11))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R11" s="2">
@@ -1495,33 +1491,33 @@
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <f>O11+P11+Q11+R11+S11</f>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:26" ht="22.5" hidden="1">
+    <row r="12" spans="1:27" ht="22.5">
       <c r="A12" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J12" s="2">
         <v>8</v>
@@ -1539,7 +1535,7 @@
         <v>21</v>
       </c>
       <c r="Q12" s="2">
-        <f>ROUND(MAX(0,IF(W12="",0,(VLOOKUP(W12,$B$2:$T$41,19,FALSE)-(O12+P12+R12+S12))/X12),IF(AND(A12="Infantry",ISERROR(SEARCH("Confined",E12))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O12+P12+R12+S12))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R12" s="2">
@@ -1549,33 +1545,33 @@
         <v>0</v>
       </c>
       <c r="T12" s="2">
-        <f>O12+P12+Q12+R12+S12</f>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:26" ht="33.75" hidden="1">
+    <row r="13" spans="1:27" ht="33.75">
       <c r="A13" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J13" s="2">
         <v>8</v>
@@ -1593,7 +1589,7 @@
         <v>21</v>
       </c>
       <c r="Q13" s="2">
-        <f>ROUND(MAX(0,IF(W13="",0,(VLOOKUP(W13,$B$2:$T$41,19,FALSE)-(O13+P13+R13+S13))/X13),IF(AND(A13="Infantry",ISERROR(SEARCH("Confined",E13))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O13+P13+R13+S13))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R13" s="2">
@@ -1603,32 +1599,32 @@
         <v>0</v>
       </c>
       <c r="T13" s="2">
-        <f>O13+P13+Q13+R13+S13</f>
+        <f t="shared" si="1"/>
         <v>21</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:26" ht="33.75" hidden="1">
+    <row r="14" spans="1:27" ht="33.75">
       <c r="A14" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2">
@@ -1647,7 +1643,7 @@
         <v>17</v>
       </c>
       <c r="Q14" s="2">
-        <f>ROUND(MAX(0,IF(W14="",0,(VLOOKUP(W14,$B$2:$T$41,19,FALSE)-(O14+P14+R14+S14))/X14),IF(AND(A14="Infantry",ISERROR(SEARCH("Confined",E14))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O14+P14+R14+S14))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R14" s="2">
@@ -1657,31 +1653,31 @@
         <v>0</v>
       </c>
       <c r="T14" s="2">
-        <f>O14+P14+Q14+R14+S14</f>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:26" ht="78.75" hidden="1">
+    <row r="15" spans="1:27" ht="78.75">
       <c r="A15" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
@@ -1693,10 +1689,10 @@
       </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O15" s="2">
         <v>0</v>
@@ -1705,7 +1701,7 @@
         <v>1</v>
       </c>
       <c r="Q15" s="2">
-        <f>ROUND(MAX(0,IF(W15="",0,(VLOOKUP(W15,$B$2:$T$41,19,FALSE)-(O15+P15+R15+S15))/X15),IF(AND(A15="Infantry",ISERROR(SEARCH("Confined",E15))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O15+P15+R15+S15))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>17</v>
       </c>
       <c r="R15" s="2">
@@ -1715,7 +1711,7 @@
         <v>-1</v>
       </c>
       <c r="T15" s="2">
-        <f>O15+P15+Q15+R15+S15</f>
+        <f t="shared" si="1"/>
         <v>17</v>
       </c>
       <c r="U15" s="2">
@@ -1723,31 +1719,31 @@
       </c>
       <c r="V15" s="2"/>
       <c r="W15" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="X15" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="78.75" hidden="1">
+    <row r="16" spans="1:27" ht="78.75">
       <c r="A16" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -1759,10 +1755,10 @@
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O16" s="2">
         <v>0</v>
@@ -1771,7 +1767,7 @@
         <v>4</v>
       </c>
       <c r="Q16" s="2">
-        <f>ROUND(MAX(0,IF(W16="",0,(VLOOKUP(W16,$B$2:$T$41,19,FALSE)-(O16+P16+R16+S16))/X16),IF(AND(A16="Infantry",ISERROR(SEARCH("Confined",E16))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O16+P16+R16+S16))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>13</v>
       </c>
       <c r="R16" s="2">
@@ -1781,7 +1777,7 @@
         <v>-1</v>
       </c>
       <c r="T16" s="2">
-        <f>O16+P16+Q16+R16+S16</f>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="U16" s="2">
@@ -1789,29 +1785,29 @@
       </c>
       <c r="V16" s="2"/>
       <c r="W16" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="X16" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="22.5" hidden="1">
+    <row r="17" spans="1:24" ht="22.5">
       <c r="A17" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1831,7 +1827,7 @@
         <v>14</v>
       </c>
       <c r="Q17" s="2">
-        <f>ROUND(MAX(0,IF(W17="",0,(VLOOKUP(W17,$B$2:$T$41,19,FALSE)-(O17+P17+R17+S17))/X17),IF(AND(A17="Infantry",ISERROR(SEARCH("Confined",E17))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O17+P17+R17+S17))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R17" s="2">
@@ -1841,33 +1837,33 @@
         <v>0</v>
       </c>
       <c r="T17" s="2">
-        <f>O17+P17+Q17+R17+S17</f>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:26" ht="157.5">
+    <row r="18" spans="1:24" ht="157.5">
       <c r="A18" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J18" s="2">
         <v>8</v>
@@ -1885,7 +1881,7 @@
         <v>12</v>
       </c>
       <c r="Q18" s="2">
-        <f>ROUND(MAX(0,IF(W18="",0,(VLOOKUP(W18,$B$2:$T$41,19,FALSE)-(O18+P18+R18+S18))/X18),IF(AND(A18="Infantry",ISERROR(SEARCH("Confined",E18))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O18+P18+R18+S18))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R18" s="2">
@@ -1895,7 +1891,7 @@
         <v>0</v>
       </c>
       <c r="T18" s="2">
-        <f>O18+P18+Q18+R18+S18</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="U18" s="2">
@@ -1903,26 +1899,26 @@
       </c>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:26" ht="45" hidden="1">
+    <row r="19" spans="1:24" ht="45">
       <c r="A19" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2">
@@ -1941,7 +1937,7 @@
         <v>13</v>
       </c>
       <c r="Q19" s="2">
-        <f>ROUND(MAX(0,IF(W19="",0,(VLOOKUP(W19,$B$2:$T$41,19,FALSE)-(O19+P19+R19+S19))/X19),IF(AND(A19="Infantry",ISERROR(SEARCH("Confined",E19))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O19+P19+R19+S19))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R19" s="2">
@@ -1951,29 +1947,29 @@
         <v>-1</v>
       </c>
       <c r="T19" s="2">
-        <f>O19+P19+Q19+R19+S19</f>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:26" ht="112.5" hidden="1">
+    <row r="20" spans="1:24" ht="112.5">
       <c r="A20" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -1993,7 +1989,7 @@
         <v>14</v>
       </c>
       <c r="Q20" s="2">
-        <f>ROUND(MAX(0,IF(W20="",0,(VLOOKUP(W20,$B$2:$T$41,19,FALSE)-(O20+P20+R20+S20))/X20),IF(AND(A20="Infantry",ISERROR(SEARCH("Confined",E20))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O20+P20+R20+S20))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R20" s="2">
@@ -2003,35 +1999,35 @@
         <v>-4</v>
       </c>
       <c r="T20" s="2">
-        <f>O20+P20+Q20+R20+S20</f>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:26" ht="112.5" hidden="1">
+    <row r="21" spans="1:24" ht="112.5">
       <c r="A21" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J21" s="2">
         <v>4</v>
@@ -2049,7 +2045,7 @@
         <v>10</v>
       </c>
       <c r="Q21" s="2">
-        <f>ROUND(MAX(0,IF(W21="",0,(VLOOKUP(W21,$B$2:$T$41,19,FALSE)-(O21+P21+R21+S21))/X21),IF(AND(A21="Infantry",ISERROR(SEARCH("Confined",E21))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O21+P21+R21+S21))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R21" s="2">
@@ -2059,7 +2055,7 @@
         <v>-2</v>
       </c>
       <c r="T21" s="2">
-        <f>O21+P21+Q21+R21+S21</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="U21" s="2">
@@ -2067,25 +2063,25 @@
       </c>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:26" ht="22.5">
+    <row r="22" spans="1:24" ht="22.5">
       <c r="A22" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J22" s="2">
         <v>8</v>
@@ -2103,7 +2099,7 @@
         <v>8</v>
       </c>
       <c r="Q22" s="2">
-        <f>ROUND(MAX(0,IF(W22="",0,(VLOOKUP(W22,$B$2:$T$41,19,FALSE)-(O22+P22+R22+S22))/X22),IF(AND(A22="Infantry",ISERROR(SEARCH("Confined",E22))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O22+P22+R22+S22))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R22" s="2">
@@ -2113,31 +2109,31 @@
         <v>0</v>
       </c>
       <c r="T22" s="2">
-        <f>O22+P22+Q22+R22+S22</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:26" ht="22.5">
+    <row r="23" spans="1:24" ht="22.5">
       <c r="A23" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J23" s="2">
         <v>8</v>
@@ -2155,7 +2151,7 @@
         <v>8</v>
       </c>
       <c r="Q23" s="2">
-        <f>ROUND(MAX(0,IF(W23="",0,(VLOOKUP(W23,$B$2:$T$41,19,FALSE)-(O23+P23+R23+S23))/X23),IF(AND(A23="Infantry",ISERROR(SEARCH("Confined",E23))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O23+P23+R23+S23))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R23" s="2">
@@ -2165,31 +2161,31 @@
         <v>0</v>
       </c>
       <c r="T23" s="2">
-        <f>O23+P23+Q23+R23+S23</f>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
     </row>
-    <row r="24" spans="1:26" ht="123.75" hidden="1">
+    <row r="24" spans="1:24" ht="123.75">
       <c r="A24" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -2200,13 +2196,13 @@
         <v>1</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O24" s="2">
         <v>0</v>
@@ -2215,7 +2211,7 @@
         <v>3</v>
       </c>
       <c r="Q24" s="2">
-        <f>ROUND(MAX(0,IF(W24="",0,(VLOOKUP(W24,$B$2:$T$41,19,FALSE)-(O24+P24+R24+S24))/X24),IF(AND(A24="Infantry",ISERROR(SEARCH("Confined",E24))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O24+P24+R24+S24))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>4</v>
       </c>
       <c r="R24" s="2">
@@ -2225,7 +2221,7 @@
         <v>-1</v>
       </c>
       <c r="T24" s="2">
-        <f>O24+P24+Q24+R24+S24</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U24" s="2">
@@ -2233,37 +2229,37 @@
       </c>
       <c r="V24" s="2"/>
       <c r="W24" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="X24" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="112.5" hidden="1">
+    <row r="25" spans="1:24" ht="112.5">
       <c r="A25" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J25" s="2">
         <v>8</v>
@@ -2281,7 +2277,7 @@
         <v>8</v>
       </c>
       <c r="Q25" s="2">
-        <f>ROUND(MAX(0,IF(W25="",0,(VLOOKUP(W25,$B$2:$T$41,19,FALSE)-(O25+P25+R25+S25))/X25),IF(AND(A25="Infantry",ISERROR(SEARCH("Confined",E25))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O25+P25+R25+S25))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R25" s="2">
@@ -2291,7 +2287,7 @@
         <v>-1</v>
       </c>
       <c r="T25" s="2">
-        <f>O25+P25+Q25+R25+S25</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U25" s="2">
@@ -2299,27 +2295,27 @@
       </c>
       <c r="V25" s="2"/>
     </row>
-    <row r="26" spans="1:26" ht="45">
+    <row r="26" spans="1:24" ht="45">
       <c r="A26" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J26" s="2">
         <v>8</v>
@@ -2337,7 +2333,7 @@
         <v>8</v>
       </c>
       <c r="Q26" s="2">
-        <f>ROUND(MAX(0,IF(W26="",0,(VLOOKUP(W26,$B$2:$T$41,19,FALSE)-(O26+P26+R26+S26))/X26),IF(AND(A26="Infantry",ISERROR(SEARCH("Confined",E26))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O26+P26+R26+S26))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R26" s="2">
@@ -2347,33 +2343,33 @@
         <v>-1</v>
       </c>
       <c r="T26" s="2">
-        <f>O26+P26+Q26+R26+S26</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:26" ht="90">
+    <row r="27" spans="1:24" ht="90">
       <c r="A27" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J27" s="2">
         <v>8</v>
@@ -2391,7 +2387,7 @@
         <v>8</v>
       </c>
       <c r="Q27" s="2">
-        <f>ROUND(MAX(0,IF(W27="",0,(VLOOKUP(W27,$B$2:$T$41,19,FALSE)-(O27+P27+R27+S27))/X27),IF(AND(A27="Infantry",ISERROR(SEARCH("Confined",E27))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O27+P27+R27+S27))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R27" s="2">
@@ -2401,7 +2397,7 @@
         <v>-1</v>
       </c>
       <c r="T27" s="2">
-        <f>O27+P27+Q27+R27+S27</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U27" s="2">
@@ -2409,28 +2405,28 @@
       </c>
       <c r="V27" s="2"/>
     </row>
-    <row r="28" spans="1:26" ht="101.25">
+    <row r="28" spans="1:24" ht="101.25">
       <c r="A28" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2">
@@ -2449,7 +2445,7 @@
         <v>8</v>
       </c>
       <c r="Q28" s="2">
-        <f>ROUND(MAX(0,IF(W28="",0,(VLOOKUP(W28,$B$2:$T$41,19,FALSE)-(O28+P28+R28+S28))/X28),IF(AND(A28="Infantry",ISERROR(SEARCH("Confined",E28))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O28+P28+R28+S28))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R28" s="2">
@@ -2459,7 +2455,7 @@
         <v>-1</v>
       </c>
       <c r="T28" s="2">
-        <f>O28+P28+Q28+R28+S28</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U28" s="2">
@@ -2467,28 +2463,28 @@
       </c>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:26" ht="33.75" hidden="1">
+    <row r="29" spans="1:24" ht="33.75">
       <c r="A29" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2">
@@ -2498,7 +2494,7 @@
         <v>1</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -2509,7 +2505,7 @@
         <v>8</v>
       </c>
       <c r="Q29" s="2">
-        <f>ROUND(MAX(0,IF(W29="",0,(VLOOKUP(W29,$B$2:$T$41,19,FALSE)-(O29+P29+R29+S29))/X29),IF(AND(A29="Infantry",ISERROR(SEARCH("Confined",E29))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O29+P29+R29+S29))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R29" s="2">
@@ -2519,7 +2515,7 @@
         <v>-2</v>
       </c>
       <c r="T29" s="2">
-        <f>O29+P29+Q29+R29+S29</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U29" s="2"/>
@@ -2527,26 +2523,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="22.5" hidden="1">
+    <row r="30" spans="1:24" ht="22.5">
       <c r="A30" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2">
@@ -2565,7 +2561,7 @@
         <v>5</v>
       </c>
       <c r="Q30" s="2">
-        <f>ROUND(MAX(0,IF(W30="",0,(VLOOKUP(W30,$B$2:$T$41,19,FALSE)-(O30+P30+R30+S30))/X30),IF(AND(A30="Infantry",ISERROR(SEARCH("Confined",E30))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O30+P30+R30+S30))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R30" s="2">
@@ -2575,36 +2571,36 @@
         <v>0</v>
       </c>
       <c r="T30" s="2">
-        <f>O30+P30+Q30+R30+S30</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
     </row>
-    <row r="31" spans="1:26" ht="90" hidden="1">
+    <row r="31" spans="1:24" ht="90">
       <c r="A31" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G31" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>113</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2">
@@ -2614,7 +2610,7 @@
         <v>1</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -2625,7 +2621,7 @@
         <v>5</v>
       </c>
       <c r="Q31" s="2">
-        <f>ROUND(MAX(0,IF(W31="",0,(VLOOKUP(W31,$B$2:$T$41,19,FALSE)-(O31+P31+R31+S31))/X31),IF(AND(A31="Infantry",ISERROR(SEARCH("Confined",E31))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O31+P31+R31+S31))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R31" s="2">
@@ -2635,7 +2631,7 @@
         <v>-1</v>
       </c>
       <c r="T31" s="2">
-        <f>O31+P31+Q31+R31+S31</f>
+        <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="U31" s="2">
@@ -2645,23 +2641,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:26" hidden="1">
+    <row r="32" spans="1:24">
       <c r="A32" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2681,7 +2677,7 @@
         <v>4</v>
       </c>
       <c r="Q32" s="2">
-        <f>ROUND(MAX(0,IF(W32="",0,(VLOOKUP(W32,$B$2:$T$41,19,FALSE)-(O32+P32+R32+S32))/X32),IF(AND(A32="Infantry",ISERROR(SEARCH("Confined",E32))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O32+P32+R32+S32))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R32" s="2">
@@ -2691,32 +2687,32 @@
         <v>0</v>
       </c>
       <c r="T32" s="2">
-        <f>O32+P32+Q32+R32+S32</f>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:26" ht="45" hidden="1">
+    <row r="33" spans="1:24" ht="45">
       <c r="A33" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2">
@@ -2735,7 +2731,7 @@
         <v>4</v>
       </c>
       <c r="Q33" s="2">
-        <f>ROUND(MAX(0,IF(W33="",0,(VLOOKUP(W33,$B$2:$T$41,19,FALSE)-(O33+P33+R33+S33))/X33),IF(AND(A33="Infantry",ISERROR(SEARCH("Confined",E33))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O33+P33+R33+S33))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R33" s="2">
@@ -2745,31 +2741,31 @@
         <v>-1</v>
       </c>
       <c r="T33" s="2">
-        <f>O33+P33+Q33+R33+S33</f>
+        <f t="shared" si="1"/>
         <v>5</v>
       </c>
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
     </row>
-    <row r="34" spans="1:26" ht="22.5">
+    <row r="34" spans="1:24" ht="22.5">
       <c r="A34" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J34" s="2">
         <v>8</v>
@@ -2787,7 +2783,7 @@
         <v>4</v>
       </c>
       <c r="Q34" s="2">
-        <f>ROUND(MAX(0,IF(W34="",0,(VLOOKUP(W34,$B$2:$T$41,19,FALSE)-(O34+P34+R34+S34))/X34),IF(AND(A34="Infantry",ISERROR(SEARCH("Confined",E34))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O34+P34+R34+S34))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R34" s="2">
@@ -2797,31 +2793,31 @@
         <v>0</v>
       </c>
       <c r="T34" s="2">
-        <f>O34+P34+Q34+R34+S34</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="U34" s="2"/>
       <c r="V34" s="2"/>
     </row>
-    <row r="35" spans="1:26" ht="78.75" hidden="1">
+    <row r="35" spans="1:24" ht="78.75">
       <c r="A35" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -2833,10 +2829,10 @@
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="O35" s="2">
         <v>0</v>
@@ -2845,7 +2841,7 @@
         <v>3</v>
       </c>
       <c r="Q35" s="2">
-        <f>ROUND(MAX(0,IF(W35="",0,(VLOOKUP(W35,$B$2:$T$41,19,FALSE)-(O35+P35+R35+S35))/X35),IF(AND(A35="Infantry",ISERROR(SEARCH("Confined",E35))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O35+P35+R35+S35))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R35" s="2">
@@ -2855,7 +2851,7 @@
         <v>-1</v>
       </c>
       <c r="T35" s="2">
-        <f>O35+P35+Q35+R35+S35</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="U35" s="2">
@@ -2863,33 +2859,33 @@
       </c>
       <c r="V35" s="2"/>
       <c r="W35" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="X35" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:26" ht="157.5" hidden="1">
+    <row r="36" spans="1:24" ht="157.5">
       <c r="A36" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2909,7 +2905,7 @@
         <v>3</v>
       </c>
       <c r="Q36" s="2">
-        <f>ROUND(MAX(0,IF(W36="",0,(VLOOKUP(W36,$B$2:$T$41,19,FALSE)-(O36+P36+R36+S36))/X36),IF(AND(A36="Infantry",ISERROR(SEARCH("Confined",E36))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O36+P36+R36+S36))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>2</v>
       </c>
       <c r="R36" s="2">
@@ -2919,7 +2915,7 @@
         <v>-1</v>
       </c>
       <c r="T36" s="2">
-        <f>O36+P36+Q36+R36+S36</f>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="U36" s="2">
@@ -2929,29 +2925,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:26" ht="45">
+    <row r="37" spans="1:24" ht="45">
       <c r="A37" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J37" s="2">
         <v>4</v>
@@ -2969,7 +2965,7 @@
         <v>4</v>
       </c>
       <c r="Q37" s="2">
-        <f>ROUND(MAX(0,IF(W37="",0,(VLOOKUP(W37,$B$2:$T$41,19,FALSE)-(O37+P37+R37+S37))/X37),IF(AND(A37="Infantry",ISERROR(SEARCH("Confined",E37))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O37+P37+R37+S37))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R37" s="2">
@@ -2979,35 +2975,35 @@
         <v>-2</v>
       </c>
       <c r="T37" s="2">
-        <f>O37+P37+Q37+R37+S37</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
     </row>
-    <row r="38" spans="1:26" ht="56.25">
+    <row r="38" spans="1:24" ht="56.25">
       <c r="A38" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J38" s="2">
         <v>4</v>
@@ -3025,7 +3021,7 @@
         <v>4</v>
       </c>
       <c r="Q38" s="2">
-        <f>ROUND(MAX(0,IF(W38="",0,(VLOOKUP(W38,$B$2:$T$41,19,FALSE)-(O38+P38+R38+S38))/X38),IF(AND(A38="Infantry",ISERROR(SEARCH("Confined",E38))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O38+P38+R38+S38))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R38" s="2">
@@ -3035,37 +3031,37 @@
         <v>-2</v>
       </c>
       <c r="T38" s="2">
-        <f>O38+P38+Q38+R38+S38</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
     </row>
-    <row r="39" spans="1:26" ht="101.25">
+    <row r="39" spans="1:24" ht="101.25">
       <c r="A39" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J39" s="2">
         <v>4</v>
@@ -3083,7 +3079,7 @@
         <v>4</v>
       </c>
       <c r="Q39" s="2">
-        <f>ROUND(MAX(0,IF(W39="",0,(VLOOKUP(W39,$B$2:$T$41,19,FALSE)-(O39+P39+R39+S39))/X39),IF(AND(A39="Infantry",ISERROR(SEARCH("Confined",E39))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O39+P39+R39+S39))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R39" s="2">
@@ -3093,7 +3089,7 @@
         <v>-2</v>
       </c>
       <c r="T39" s="2">
-        <f>O39+P39+Q39+R39+S39</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="U39" s="2">
@@ -3103,29 +3099,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:26" ht="56.25">
+    <row r="40" spans="1:24" ht="56.25">
       <c r="A40" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J40" s="2">
         <v>4</v>
@@ -3143,7 +3139,7 @@
         <v>4</v>
       </c>
       <c r="Q40" s="2">
-        <f>ROUND(MAX(0,IF(W40="",0,(VLOOKUP(W40,$B$2:$T$41,19,FALSE)-(O40+P40+R40+S40))/X40),IF(AND(A40="Infantry",ISERROR(SEARCH("Confined",E40))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O40+P40+R40+S40))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R40" s="2">
@@ -3153,32 +3149,32 @@
         <v>-2</v>
       </c>
       <c r="T40" s="2">
-        <f>O40+P40+Q40+R40+S40</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
     </row>
-    <row r="41" spans="1:26" ht="33.75" hidden="1">
+    <row r="41" spans="1:24" ht="33.75">
       <c r="A41" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2">
@@ -3197,7 +3193,7 @@
         <v>4</v>
       </c>
       <c r="Q41" s="2">
-        <f>ROUND(MAX(0,IF(W41="",0,(VLOOKUP(W41,$B$2:$T$41,19,FALSE)-(O41+P41+R41+S41))/X41),IF(AND(A41="Infantry",ISERROR(SEARCH("Confined",E41))),(VLOOKUP(FarEdgeTarget,$B$2:$T$41,19,FALSE)-(O41+P41+R41+S41))/FarEdgeDistance,0))*PremiumFactor,0)</f>
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R41" s="2">
@@ -3207,7 +3203,7 @@
         <v>-2</v>
       </c>
       <c r="T41" s="2">
-        <f>O41+P41+Q41+R41+S41</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="U41" s="2"/>
@@ -3216,13 +3212,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X41">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Cavalry / Leaper"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:X41"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
The pieces spreadsheet as the designer last left it
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="138">
   <si>
     <t>Piece Class</t>
   </si>
@@ -825,6 +825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -913,7 +914,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="2" spans="1:27" ht="33.75">
+    <row r="2" spans="1:27" ht="33.75" hidden="1">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -973,7 +974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="33.75">
+    <row r="3" spans="1:27" ht="33.75" hidden="1">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1035,7 +1036,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="22.5">
+    <row r="4" spans="1:27" ht="22.5" hidden="1">
       <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
@@ -1097,7 +1098,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="33.75">
+    <row r="5" spans="1:27" ht="33.75" hidden="1">
       <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
@@ -1155,10 +1156,8 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="33.75">
-      <c r="A6" s="5" t="s">
-        <v>20</v>
-      </c>
+    <row r="6" spans="1:27" ht="33.75" hidden="1">
+      <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
         <v>30</v>
       </c>
@@ -1215,7 +1214,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="33.75">
+    <row r="7" spans="1:27" ht="33.75" hidden="1">
       <c r="A7" s="5" t="s">
         <v>20</v>
       </c>
@@ -1269,7 +1268,7 @@
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
     </row>
-    <row r="8" spans="1:27" ht="78.75">
+    <row r="8" spans="1:27" ht="78.75" hidden="1">
       <c r="A8" s="5" t="s">
         <v>20</v>
       </c>
@@ -1333,7 +1332,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="33.75">
+    <row r="9" spans="1:27" ht="33.75" hidden="1">
       <c r="A9" s="5" t="s">
         <v>22</v>
       </c>
@@ -1389,7 +1388,7 @@
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
     </row>
-    <row r="10" spans="1:27" ht="22.5">
+    <row r="10" spans="1:27" ht="22.5" hidden="1">
       <c r="A10" s="5" t="s">
         <v>22</v>
       </c>
@@ -1443,7 +1442,7 @@
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
     </row>
-    <row r="11" spans="1:27" ht="33.75">
+    <row r="11" spans="1:27" ht="33.75" hidden="1">
       <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
@@ -1497,7 +1496,7 @@
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:27" ht="22.5">
+    <row r="12" spans="1:27" ht="22.5" hidden="1">
       <c r="A12" s="5" t="s">
         <v>22</v>
       </c>
@@ -1551,7 +1550,7 @@
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:27" ht="33.75">
+    <row r="13" spans="1:27" ht="33.75" hidden="1">
       <c r="A13" s="5" t="s">
         <v>22</v>
       </c>
@@ -1605,7 +1604,7 @@
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:27" ht="33.75">
+    <row r="14" spans="1:27" ht="33.75" hidden="1">
       <c r="A14" s="5" t="s">
         <v>22</v>
       </c>
@@ -1725,7 +1724,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:27" ht="78.75">
+    <row r="16" spans="1:27" ht="78.75" hidden="1">
       <c r="A16" s="5" t="s">
         <v>22</v>
       </c>
@@ -1791,7 +1790,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:24" ht="22.5">
+    <row r="17" spans="1:24" ht="22.5" hidden="1">
       <c r="A17" s="5" t="s">
         <v>22</v>
       </c>
@@ -1843,7 +1842,7 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:24" ht="157.5">
+    <row r="18" spans="1:24" ht="157.5" hidden="1">
       <c r="A18" s="5" t="s">
         <v>23</v>
       </c>
@@ -1899,7 +1898,7 @@
       </c>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:24" ht="45">
+    <row r="19" spans="1:24" ht="45" hidden="1">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -1953,7 +1952,7 @@
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:24" ht="112.5">
+    <row r="20" spans="1:24" ht="112.5" hidden="1">
       <c r="A20" s="5" t="s">
         <v>24</v>
       </c>
@@ -2005,7 +2004,7 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:24" ht="112.5">
+    <row r="21" spans="1:24" ht="112.5" hidden="1">
       <c r="A21" s="5" t="s">
         <v>24</v>
       </c>
@@ -2063,7 +2062,7 @@
       </c>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:24" ht="22.5">
+    <row r="22" spans="1:24" ht="22.5" hidden="1">
       <c r="A22" s="5" t="s">
         <v>23</v>
       </c>
@@ -2115,7 +2114,7 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:24" ht="22.5">
+    <row r="23" spans="1:24" ht="22.5" hidden="1">
       <c r="A23" s="5" t="s">
         <v>23</v>
       </c>
@@ -2235,7 +2234,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="112.5">
+    <row r="25" spans="1:24" ht="112.5" hidden="1">
       <c r="A25" s="5" t="s">
         <v>24</v>
       </c>
@@ -2295,7 +2294,7 @@
       </c>
       <c r="V25" s="2"/>
     </row>
-    <row r="26" spans="1:24" ht="45">
+    <row r="26" spans="1:24" ht="45" hidden="1">
       <c r="A26" s="5" t="s">
         <v>23</v>
       </c>
@@ -2349,7 +2348,7 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:24" ht="90">
+    <row r="27" spans="1:24" ht="90" hidden="1">
       <c r="A27" s="5" t="s">
         <v>23</v>
       </c>
@@ -2405,7 +2404,7 @@
       </c>
       <c r="V27" s="2"/>
     </row>
-    <row r="28" spans="1:24" ht="101.25">
+    <row r="28" spans="1:24" ht="101.25" hidden="1">
       <c r="A28" s="5" t="s">
         <v>23</v>
       </c>
@@ -2463,7 +2462,7 @@
       </c>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:24" ht="33.75">
+    <row r="29" spans="1:24" ht="33.75" hidden="1">
       <c r="A29" s="5" t="s">
         <v>21</v>
       </c>
@@ -2523,7 +2522,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="22.5">
+    <row r="30" spans="1:24" ht="22.5" hidden="1">
       <c r="A30" s="5" t="s">
         <v>21</v>
       </c>
@@ -2577,7 +2576,7 @@
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
     </row>
-    <row r="31" spans="1:24" ht="90">
+    <row r="31" spans="1:24" ht="90" hidden="1">
       <c r="A31" s="5" t="s">
         <v>21</v>
       </c>
@@ -2641,7 +2640,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:24">
+    <row r="32" spans="1:24" hidden="1">
       <c r="A32" s="5" t="s">
         <v>21</v>
       </c>
@@ -2693,7 +2692,7 @@
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:24" ht="45">
+    <row r="33" spans="1:24" ht="45" hidden="1">
       <c r="A33" s="5" t="s">
         <v>21</v>
       </c>
@@ -2747,7 +2746,7 @@
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
     </row>
-    <row r="34" spans="1:24" ht="22.5">
+    <row r="34" spans="1:24" ht="22.5" hidden="1">
       <c r="A34" s="5" t="s">
         <v>23</v>
       </c>
@@ -2865,7 +2864,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="157.5">
+    <row r="36" spans="1:24" ht="157.5" hidden="1">
       <c r="A36" s="5" t="s">
         <v>21</v>
       </c>
@@ -2925,7 +2924,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="45">
+    <row r="37" spans="1:24" ht="45" hidden="1">
       <c r="A37" s="5" t="s">
         <v>23</v>
       </c>
@@ -2981,7 +2980,7 @@
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
     </row>
-    <row r="38" spans="1:24" ht="56.25">
+    <row r="38" spans="1:24" ht="56.25" hidden="1">
       <c r="A38" s="5" t="s">
         <v>23</v>
       </c>
@@ -3037,7 +3036,7 @@
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
     </row>
-    <row r="39" spans="1:24" ht="101.25">
+    <row r="39" spans="1:24" ht="101.25" hidden="1">
       <c r="A39" s="5" t="s">
         <v>23</v>
       </c>
@@ -3099,7 +3098,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:24" ht="56.25">
+    <row r="40" spans="1:24" ht="56.25" hidden="1">
       <c r="A40" s="5" t="s">
         <v>23</v>
       </c>
@@ -3155,7 +3154,7 @@
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
     </row>
-    <row r="41" spans="1:24" ht="33.75">
+    <row r="41" spans="1:24" ht="33.75" hidden="1">
       <c r="A41" s="5" t="s">
         <v>21</v>
       </c>
@@ -3212,7 +3211,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X41"/>
+  <autoFilter ref="A1:X41">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Infantry"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <customFilters and="1">
+        <customFilter val="*Pawn*"/>
+      </customFilters>
+    </filterColumn>
+  </autoFilter>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
A piece that may promote into a leader starts from a leader bonus of 50, as a leader from 60, with the rest counted on top: the Lance is 56, the Shogi Pawn 54; the spreadsheet holds the bonus as a setting, and two scripts read and set its cells
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -14,8 +14,9 @@
     <definedName name="FarEdgeDistance">Sheet1!$AA$4</definedName>
     <definedName name="FarEdgeTarget">Sheet1!$AA$3</definedName>
     <definedName name="PremiumFactor">Sheet1!$AA$2</definedName>
+    <definedName name="LeaderPromotionBonus">Sheet1!$AA$5</definedName>
   </definedNames>
-  <calcPr calcId="114210"/>
+  <calcPr fullCalcOnLoad="1" calcId="114210"/>
 </workbook>
 </file>
 
@@ -877,8 +878,10 @@
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>Leader bonus (60 for a leader; LeaderPromotionBonus for a piece that may promote into one)</t>
+        </is>
       </c>
       <c r="P1" s="3" t="s">
         <v>129</v>
@@ -1155,6 +1158,14 @@
       <c r="V5" s="2">
         <v>5</v>
       </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>LeaderPromotionBonus</t>
+        </is>
+      </c>
+      <c r="AA5" s="2">
+        <v>50</v>
+      </c>
     </row>
     <row r="6" spans="1:27" ht="33.75" hidden="1">
       <c r="A6" s="5"/>
@@ -1694,14 +1705,15 @@
         <v>121</v>
       </c>
       <c r="O15" s="2">
-        <v>0</v>
+        <f>LeaderPromotionBonus</f>
+        <v>50</v>
       </c>
       <c r="P15" s="2">
         <v>1</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="R15" s="2">
         <v>0</v>
@@ -1711,7 +1723,7 @@
       </c>
       <c r="T15" s="2">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="U15" s="2">
         <v>2</v>
@@ -1760,14 +1772,15 @@
         <v>121</v>
       </c>
       <c r="O16" s="2">
-        <v>0</v>
+        <f>LeaderPromotionBonus</f>
+        <v>50</v>
       </c>
       <c r="P16" s="2">
         <v>4</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="R16" s="2">
         <v>0</v>
@@ -1777,7 +1790,7 @@
       </c>
       <c r="T16" s="2">
         <f t="shared" si="1"/>
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="U16" s="2">
         <v>2</v>

</xml_diff>

<commit_message>
Player profiles: a player may change the name others see, and link several sign-in services to one player (with a one-time code carried through the sign-in window), or unlink any but the last; the page offers this under Profile
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Other Potential Pieces.xlsx
+++ b/docs/Other Potential Pieces.xlsx
@@ -13,15 +13,15 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$X$41</definedName>
     <definedName name="FarEdgeDistance">Sheet1!$AA$4</definedName>
     <definedName name="FarEdgeTarget">Sheet1!$AA$3</definedName>
+    <definedName name="LeaderPromotionBonus">Sheet1!$AA$5</definedName>
     <definedName name="PremiumFactor">Sheet1!$AA$2</definedName>
-    <definedName name="LeaderPromotionBonus">Sheet1!$AA$5</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1" calcId="114210"/>
+  <calcPr calcId="114210"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="139">
   <si>
     <t>Piece Class</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Promotion Condition</t>
   </si>
   <si>
-    <t>Leader bonus</t>
-  </si>
-  <si>
     <t>Special-power bonus</t>
   </si>
   <si>
@@ -435,6 +432,12 @@
   </si>
   <si>
     <t>FarEdgeDistance</t>
+  </si>
+  <si>
+    <t>Leader bonus (60 for a leader; LeaderPromotionBonus for a piece that may promote into one)</t>
+  </si>
+  <si>
+    <t>LeaderPromotionBonus</t>
   </si>
 </sst>
 </file>
@@ -826,7 +829,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AA41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -878,65 +880,63 @@
       <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="3" t="inlineStr">
-        <is>
-          <t>Leader bonus (60 for a leader; LeaderPromotionBonus for a piece that may promote into one)</t>
-        </is>
+      <c r="O1" s="3" t="s">
+        <v>137</v>
       </c>
       <c r="P1" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q1" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="T1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="V1" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W1" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="R1" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="S1" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="V1" s="3" t="s">
+      <c r="X1" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="Z1" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="AA1" s="3" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" ht="33.75">
+      <c r="A2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="W1" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="X1" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="Z1" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="AA1" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="2" spans="1:27" ht="33.75" hidden="1">
-      <c r="A2" s="5" t="s">
-        <v>20</v>
-      </c>
       <c r="B2" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2">
@@ -971,35 +971,35 @@
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
       <c r="Z2" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="AA2" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" ht="33.75" hidden="1">
+    <row r="3" spans="1:27" ht="33.75">
       <c r="A3" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J3" s="2">
         <v>8</v>
@@ -1033,32 +1033,32 @@
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
       <c r="Z3" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AA3" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" ht="22.5" hidden="1">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27" ht="22.5">
       <c r="A4" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2">
@@ -1068,7 +1068,7 @@
         <v>1</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
@@ -1095,31 +1095,31 @@
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
       <c r="Z4" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="AA4" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="33.75" hidden="1">
+    <row r="5" spans="1:27" ht="33.75">
       <c r="A5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -1130,7 +1130,7 @@
         <v>7</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="M5" s="2"/>
       <c r="N5" s="2"/>
@@ -1158,35 +1158,33 @@
       <c r="V5" s="2">
         <v>5</v>
       </c>
-      <c r="Z5" s="2" t="inlineStr">
-        <is>
-          <t>LeaderPromotionBonus</t>
-        </is>
+      <c r="Z5" s="2" t="s">
+        <v>138</v>
       </c>
       <c r="AA5" s="2">
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="33.75" hidden="1">
+    <row r="6" spans="1:27" ht="33.75">
       <c r="A6" s="5"/>
       <c r="B6" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D6" s="2"/>
       <c r="E6" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2">
@@ -1196,7 +1194,7 @@
         <v>1</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -1225,26 +1223,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="33.75" hidden="1">
+    <row r="7" spans="1:27" ht="33.75">
       <c r="A7" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2">
@@ -1279,26 +1277,26 @@
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
     </row>
-    <row r="8" spans="1:27" ht="78.75" hidden="1">
+    <row r="8" spans="1:27" ht="78.75">
       <c r="A8" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2">
@@ -1309,10 +1307,10 @@
       </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="O8" s="2">
         <v>60</v>
@@ -1337,143 +1335,169 @@
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="W8" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="X8" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:27" ht="33.75" hidden="1">
+    <row r="9" spans="1:27" ht="78.75">
       <c r="A9" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="2"/>
+        <v>85</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>111</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
       <c r="J9" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K9" s="2">
         <v>7</v>
       </c>
       <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
+      <c r="M9" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="O9" s="2">
-        <v>0</v>
+        <f ca="1">LeaderPromotionBonus</f>
+        <v>50</v>
       </c>
       <c r="P9" s="2">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R9" s="2">
+        <v>0</v>
+      </c>
+      <c r="S9" s="2">
+        <v>-1</v>
+      </c>
+      <c r="T9" s="2">
+        <f t="shared" si="1"/>
+        <v>56</v>
+      </c>
+      <c r="U9" s="2">
         <v>2</v>
       </c>
-      <c r="S9" s="2">
-        <v>0</v>
-      </c>
-      <c r="T9" s="2">
-        <f t="shared" si="1"/>
-        <v>37</v>
-      </c>
-      <c r="U9" s="2"/>
       <c r="V9" s="2"/>
-    </row>
-    <row r="10" spans="1:27" ht="22.5" hidden="1">
+      <c r="W9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X9" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" ht="78.75">
       <c r="A10" s="5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>34</v>
+        <v>60</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="2"/>
+        <v>86</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>111</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="K10" s="2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
+      <c r="M10" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>120</v>
+      </c>
       <c r="O10" s="2">
-        <v>0</v>
+        <f ca="1">LeaderPromotionBonus</f>
+        <v>50</v>
       </c>
       <c r="P10" s="2">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R10" s="2">
         <v>0</v>
       </c>
       <c r="S10" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="T10" s="2">
         <f t="shared" si="1"/>
-        <v>27</v>
-      </c>
-      <c r="U10" s="2"/>
+        <v>54</v>
+      </c>
+      <c r="U10" s="2">
+        <v>2</v>
+      </c>
       <c r="V10" s="2"/>
-    </row>
-    <row r="11" spans="1:27" ht="33.75" hidden="1">
+      <c r="W10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="X10" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" ht="33.75">
       <c r="A11" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H11" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="I11" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J11" s="2">
         <v>8</v>
@@ -1488,47 +1512,47 @@
         <v>0</v>
       </c>
       <c r="P11" s="2">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="Q11" s="2">
         <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
       <c r="R11" s="2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="S11" s="2">
         <v>0</v>
       </c>
       <c r="T11" s="2">
         <f t="shared" si="1"/>
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
     </row>
-    <row r="12" spans="1:27" ht="22.5" hidden="1">
+    <row r="12" spans="1:27" ht="22.5">
       <c r="A12" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G12" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="H12" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>111</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="I12" s="2"/>
       <c r="J12" s="2">
         <v>8</v>
       </c>
@@ -1542,7 +1566,7 @@
         <v>0</v>
       </c>
       <c r="P12" s="2">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="Q12" s="2">
         <f t="shared" ca="1" si="0"/>
@@ -1556,32 +1580,32 @@
       </c>
       <c r="T12" s="2">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
     </row>
-    <row r="13" spans="1:27" ht="33.75" hidden="1">
+    <row r="13" spans="1:27" ht="33.75">
       <c r="A13" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
-        <v>111</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J13" s="2">
         <v>8</v>
@@ -1596,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="P13" s="2">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="Q13" s="2">
         <f t="shared" ca="1" si="0"/>
@@ -1610,17 +1634,17 @@
       </c>
       <c r="T13" s="2">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
     </row>
-    <row r="14" spans="1:27" ht="33.75" hidden="1">
+    <row r="14" spans="1:27" ht="22.5">
       <c r="A14" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>75</v>
@@ -1628,15 +1652,15 @@
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>111</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="G14" s="2"/>
       <c r="H14" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="I14" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="J14" s="2">
         <v>8</v>
       </c>
@@ -1650,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="P14" s="2">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="Q14" s="2">
         <f t="shared" ca="1" si="0"/>
@@ -1664,162 +1688,136 @@
       </c>
       <c r="T14" s="2">
         <f t="shared" si="1"/>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
     </row>
-    <row r="15" spans="1:27" ht="78.75">
+    <row r="15" spans="1:27" ht="33.75">
       <c r="A15" s="5" t="s">
         <v>21</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>100</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="J15" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K15" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="L15" s="2"/>
-      <c r="M15" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>121</v>
-      </c>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
       <c r="O15" s="2">
-        <f>LeaderPromotionBonus</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P15" s="2">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="Q15" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="R15" s="2">
         <v>0</v>
       </c>
       <c r="S15" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T15" s="2">
         <f t="shared" si="1"/>
-        <v>54</v>
-      </c>
-      <c r="U15" s="2">
-        <v>2</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="U15" s="2"/>
       <c r="V15" s="2"/>
-      <c r="W15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X15" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" ht="78.75" hidden="1">
+    </row>
+    <row r="16" spans="1:27" ht="33.75">
       <c r="A16" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>96</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="H16" s="2"/>
+        <v>110</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>110</v>
+      </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="K16" s="2">
         <v>7</v>
       </c>
       <c r="L16" s="2"/>
-      <c r="M16" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="N16" s="2" t="s">
-        <v>121</v>
-      </c>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
       <c r="O16" s="2">
-        <f>LeaderPromotionBonus</f>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="P16" s="2">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="Q16" s="2">
         <f t="shared" ca="1" si="0"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="R16" s="2">
         <v>0</v>
       </c>
       <c r="S16" s="2">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="T16" s="2">
         <f t="shared" si="1"/>
-        <v>56</v>
-      </c>
-      <c r="U16" s="2">
-        <v>2</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="U16" s="2"/>
       <c r="V16" s="2"/>
-      <c r="W16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X16" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="17" spans="1:24" ht="22.5" hidden="1">
+    </row>
+    <row r="17" spans="1:24" ht="22.5">
       <c r="A17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -1855,27 +1853,27 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
     </row>
-    <row r="18" spans="1:24" ht="157.5" hidden="1">
+    <row r="18" spans="1:24" ht="157.5">
       <c r="A18" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J18" s="2">
         <v>8</v>
@@ -1911,26 +1909,26 @@
       </c>
       <c r="V18" s="2"/>
     </row>
-    <row r="19" spans="1:24" ht="45" hidden="1">
+    <row r="19" spans="1:24" ht="45">
       <c r="A19" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2">
@@ -1965,23 +1963,23 @@
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
     </row>
-    <row r="20" spans="1:24" ht="112.5" hidden="1">
+    <row r="20" spans="1:24" ht="112.5">
       <c r="A20" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -2017,29 +2015,29 @@
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
     </row>
-    <row r="21" spans="1:24" ht="112.5" hidden="1">
+    <row r="21" spans="1:24" ht="112.5">
       <c r="A21" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J21" s="2">
         <v>4</v>
@@ -2075,25 +2073,25 @@
       </c>
       <c r="V21" s="2"/>
     </row>
-    <row r="22" spans="1:24" ht="22.5" hidden="1">
+    <row r="22" spans="1:24" ht="22.5">
       <c r="A22" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J22" s="2">
         <v>8</v>
@@ -2127,25 +2125,25 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
     </row>
-    <row r="23" spans="1:24" ht="22.5" hidden="1">
+    <row r="23" spans="1:24" ht="22.5">
       <c r="A23" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J23" s="2">
         <v>8</v>
@@ -2181,23 +2179,23 @@
     </row>
     <row r="24" spans="1:24" ht="123.75">
       <c r="A24" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -2208,13 +2206,13 @@
         <v>1</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="N24" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O24" s="2">
         <v>0</v>
@@ -2241,37 +2239,37 @@
       </c>
       <c r="V24" s="2"/>
       <c r="W24" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="X24" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:24" ht="112.5" hidden="1">
+    <row r="25" spans="1:24" ht="112.5">
       <c r="A25" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J25" s="2">
         <v>8</v>
@@ -2307,27 +2305,27 @@
       </c>
       <c r="V25" s="2"/>
     </row>
-    <row r="26" spans="1:24" ht="45" hidden="1">
+    <row r="26" spans="1:24" ht="45">
       <c r="A26" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J26" s="2">
         <v>8</v>
@@ -2361,27 +2359,27 @@
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
-    <row r="27" spans="1:24" ht="90" hidden="1">
+    <row r="27" spans="1:24" ht="90">
       <c r="A27" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J27" s="2">
         <v>8</v>
@@ -2417,28 +2415,28 @@
       </c>
       <c r="V27" s="2"/>
     </row>
-    <row r="28" spans="1:24" ht="101.25" hidden="1">
+    <row r="28" spans="1:24" ht="101.25">
       <c r="A28" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I28" s="2"/>
       <c r="J28" s="2">
@@ -2475,28 +2473,28 @@
       </c>
       <c r="V28" s="2"/>
     </row>
-    <row r="29" spans="1:24" ht="33.75" hidden="1">
+    <row r="29" spans="1:24" ht="33.75">
       <c r="A29" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2">
@@ -2506,7 +2504,7 @@
         <v>1</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
@@ -2535,26 +2533,26 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:24" ht="22.5" hidden="1">
+    <row r="30" spans="1:24" ht="22.5">
       <c r="A30" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2">
@@ -2589,30 +2587,30 @@
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
     </row>
-    <row r="31" spans="1:24" ht="90" hidden="1">
+    <row r="31" spans="1:24" ht="90">
       <c r="A31" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G31" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2">
@@ -2622,7 +2620,7 @@
         <v>1</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M31" s="2"/>
       <c r="N31" s="2"/>
@@ -2653,23 +2651,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:24" hidden="1">
+    <row r="32" spans="1:24">
       <c r="A32" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2705,26 +2703,26 @@
       <c r="U32" s="2"/>
       <c r="V32" s="2"/>
     </row>
-    <row r="33" spans="1:24" ht="45" hidden="1">
+    <row r="33" spans="1:24" ht="45">
       <c r="A33" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I33" s="2"/>
       <c r="J33" s="2">
@@ -2759,25 +2757,25 @@
       <c r="U33" s="2"/>
       <c r="V33" s="2"/>
     </row>
-    <row r="34" spans="1:24" ht="22.5" hidden="1">
+    <row r="34" spans="1:24" ht="22.5">
       <c r="A34" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J34" s="2">
         <v>8</v>
@@ -2813,23 +2811,23 @@
     </row>
     <row r="35" spans="1:24" ht="78.75">
       <c r="A35" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
@@ -2841,10 +2839,10 @@
       </c>
       <c r="L35" s="2"/>
       <c r="M35" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="O35" s="2">
         <v>0</v>
@@ -2871,33 +2869,33 @@
       </c>
       <c r="V35" s="2"/>
       <c r="W35" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="X35" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:24" ht="157.5" hidden="1">
+    <row r="36" spans="1:24" ht="157.5">
       <c r="A36" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
@@ -2937,29 +2935,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:24" ht="45" hidden="1">
+    <row r="37" spans="1:24" ht="45">
       <c r="A37" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J37" s="2">
         <v>4</v>
@@ -2993,29 +2991,29 @@
       <c r="U37" s="2"/>
       <c r="V37" s="2"/>
     </row>
-    <row r="38" spans="1:24" ht="56.25" hidden="1">
+    <row r="38" spans="1:24" ht="56.25">
       <c r="A38" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J38" s="2">
         <v>4</v>
@@ -3049,31 +3047,31 @@
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
     </row>
-    <row r="39" spans="1:24" ht="101.25" hidden="1">
+    <row r="39" spans="1:24" ht="101.25">
       <c r="A39" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J39" s="2">
         <v>4</v>
@@ -3111,29 +3109,29 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:24" ht="56.25" hidden="1">
+    <row r="40" spans="1:24" ht="56.25">
       <c r="A40" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J40" s="2">
         <v>4</v>
@@ -3167,26 +3165,26 @@
       <c r="U40" s="2"/>
       <c r="V40" s="2"/>
     </row>
-    <row r="41" spans="1:24" ht="33.75" hidden="1">
+    <row r="41" spans="1:24" ht="33.75">
       <c r="A41" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="2">
@@ -3224,18 +3222,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X41">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Infantry"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="1">
-      <customFilters and="1">
-        <customFilter val="*Pawn*"/>
-      </customFilters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:X41"/>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>